<commit_message>
SEO: meta descriptions, offerCount, /login noindex, fix twitter:image 404
- Rewrite 8 thin meta descriptions (ai-compliance, ai-marketing-tools,
  contact, cookies, gdpr-compliance, login, privacy, security, terms)
- Add offerCount: '3' to both AggregateOffer JSON-LD blocks, fixing the
  Google rich-results validation error
- noindex /login (transactional page, no H1, no search value)
- Add og:image to /ai-marketing-tools and /blog/[slug] (Next.js replaces
  the layout openGraph block rather than merging it)
- Point twitter:image at the real brand asset; /twitter-image.png was a
  verified live 404, blanking every X/Twitter share card
- Add docs/2026-08-23-ahrefs-ads-gtm-audit.md and KB sections 47-49
</commit_message>
<xml_diff>
--- a/docs/testing/Automated-Regression-Test-Suite.xlsx
+++ b/docs/testing/Automated-Regression-Test-Suite.xlsx
@@ -1452,7 +1452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E84"/>
+  <dimension ref="A1:E98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3730,6 +3730,384 @@
         </is>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" s="10" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B85" s="10" t="inlineStr">
+        <is>
+          <t>AUTO-001</t>
+        </is>
+      </c>
+      <c r="C85" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D85" s="11" t="inlineStr">
+        <is>
+          <t>Repo: grep -rniE '24.{0,15}(tools|apps)' across app/, components/, lib/ returned one match, lib/email.ts:217, which is a false positive on the CSS fragment 'margin: 0 0 24px 0;"&gt;Tools marked FREE' -- not a tool-count claim. Every real numeric tool claim in source is 12 (layout.tsx, page.tsx, seo-config.ts, email.ts, contact/page.tsx, ai-marketing-tools/page.tsx, Pricing.tsx, Hero.tsx, CTASection.tsx, Sidebar.tsx, ToolPage.tsx, billing/page.tsx). lib/tools/registry.ts TOOLS export has exactly 12 top-level entries. Live raw HTML fetched via the connected Chrome session: homepage, /ai-marketing-tools and /contact all return zero matches for the 24-tools pattern; homepage renders '12 AI-Powered Marketing Tools', '12 Tools, One Platform' and 12 tool cards; /ai-marketing-tools renders '12 AI-Powered Marketing Tools' / '12 Tools Across 4 Categories' / 'Choose from 12 tools'; /contact renders '12 Tools, One Platform' and 'Standard: $29/mo, all 12 tools'.</t>
+        </is>
+      </c>
+      <c r="E85" s="10" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="10" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B86" s="10" t="inlineStr">
+        <is>
+          <t>AUTO-002</t>
+        </is>
+      </c>
+      <c r="C86" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D86" s="11" t="inlineStr">
+        <is>
+          <t>RESOLVED -- the 34-day live regression first logged 2026-08-11 and still failing 2026-08-22 is fixed as of this run. https://www.shijo.ai/ai-marketing-tools now serves the correct pricing table: Free $0 / Standard $29 / Pro $199 / Enterprise 'Coming Soon' with a Contact Us CTA. Raw-HTML scan of that page for '$99', '"99"' and '&gt;99&lt;' returns zero matches; homepage and /contact likewise zero. Distinct live prices on homepage: $0, $29, $278 (annual Standard, = 29*12*0.8), $199 -- all reconcile to lib/stripe/products.ts PLAN_FEATURES. Repo grep '$99' across app/, components/, lib/ = zero matches. The JSON-LD AggregateOffer highPrice is now '199' (was hardcoded '99') on both app/page.tsx and app/ai-marketing-tools/page.tsx in source AND confirmed live in the rendered ld+json on both pages. Fixes shipped in commits 963924f ('fix retired JSON-LD price') and 7a0a787; HEAD == origin/main == 7a0a787, so everything checked here is pushed and deployed. Note for context: the working tree has 47 uncommitted modified files, but a spot-diff shows these are mostly CRLF line-ending churn plus a few unshipped metadata edits (e.g. app/contact/page.tsx description) -- none of them affect pricing, and live /contact still serves the committed description, confirming the local diff is not deployed.</t>
+        </is>
+      </c>
+      <c r="E86" s="10" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B87" s="7" t="inlineStr">
+        <is>
+          <t>AUTO-003</t>
+        </is>
+      </c>
+      <c r="C87" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="D87" s="6" t="inlineStr">
+        <is>
+          <t>CRITICAL. (a) RESOLVED live: /ai-marketing-tools now names the $29 tier 'Standard' and the $199 tier 'Pro', matching PLAN_DISPLAY_NAME and matching the homepage and /contact. Card headings extracted from live raw HTML on /ai-marketing-tools are exactly Free / Standard / Pro / Enterprise; homepage the same; /contact reads 'Standard: $29/mo' and 'Pro: $199/mo'. Zero occurrences of the raw internal key 'growth' in any public page's HTML (the single homepage hit for 'Growth' is the section heading 'Choose Your Growth Plan', an ordinary English word, not a leaked tier key). (b) STILL FAILING, unchanged since first logged 2026-08-22: app/api/stripe/create-checkout/route.ts:81 returns `You are already on the ${plan} plan` interpolating the RAW internal key, and app/dashboard/billing/page.tsx:108 assigns data.error to state which line 181 renders verbatim into the visible red error banner. Net effect: a customer on the $199 tier who re-clicks upgrade is shown 'You are already on the growth plan' -- a tier name that appears nowhere in the product. Fix is one line: PLAN_DISPLAY_NAME[plan]. All other user-facing plan-name surfaces remain correct (admin/users, dashboard/billing x3, dashboard/page, dashboard/settings, UsageMeter all import PLAN_DISPLAY_NAME). The live dashboard billing HTML still cannot be diffed unauthenticated -- it correctly 30x-redirects to /login -- so (b) is verified at code level only.</t>
+        </is>
+      </c>
+      <c r="E87" s="7" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B88" s="9" t="inlineStr">
+        <is>
+          <t>AUTO-004</t>
+        </is>
+      </c>
+      <c r="C88" s="9" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="D88" s="8" t="inlineStr">
+        <is>
+          <t>Could not run -- THIRD consecutive scheduled run blocked (also blocked 2026-08-11 and 2026-08-22). No Stripe MCP tools exist in this session: ToolSearch for 'stripe products prices subscriptions' returned 'No matching deferred tools found', and mcp-registry list_connectors returned an empty connector list, i.e. no connectors are installed at all. Stripe Product .name drift is therefore unverified for 32 days (last passing run 2026-07-22). What needs checking when the connector is reconnected: prod_UAltLAeJGLVSqI (price_1TCQLpHTpiuftGGEZWt9UJ2Y, $29) must read 'SHIJO.AI Standard', and prod_UuvJvC2ZKysgfK (price_1Tv5SpHTpiuftGGEMu4TdOzs, $199) must read 'SHIJO.AI Pro'. This is the check that caught the live 'Shijo Pro' mislabel on 2026-07-19 and it is invisible to code review, since the Product name lives only in Stripe. Recommend reconnecting the Stripe connector before the next scheduled run.</t>
+        </is>
+      </c>
+      <c r="E88" s="9" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="10" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B89" s="10" t="inlineStr">
+        <is>
+          <t>AUTO-005</t>
+        </is>
+      </c>
+      <c r="C89" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D89" s="11" t="inlineStr">
+        <is>
+          <t>Ran live against https://www.shijo.ai/api/auth/register. The sandbox HTTP proxy still refuses direct curl to shijo.ai (403 from proxy after CONNECT), so this was executed as a same-origin fetch with credentials:'omit' from the connected Chrome session on the live origin. POST {name:'Reg Test', email:'not-a-valid-email', password:'ValidPass123!', confirmPassword:'ValidPass123!'} returned HTTP 400 with body {"error":"Please enter a valid email address"}. Server-side email-format validation holds against a direct API call that bypasses the client form. No account created.</t>
+        </is>
+      </c>
+      <c r="E89" s="10" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="10" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B90" s="10" t="inlineStr">
+        <is>
+          <t>AUTO-006</t>
+        </is>
+      </c>
+      <c r="C90" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D90" s="11" t="inlineStr">
+        <is>
+          <t>Live POST to /api/auth/register (same same-origin fetch method as AUTO-005) with email shijo-regtest-mismatch-20260823@mailinator.com, password 'ValidPass123!' vs confirmPassword 'DifferentPass456!' returned HTTP 400 with body {"error":"Passwords do not match"}. The server-side mismatch check shipped 2026-07-19 remains live. Throwaway mailinator address used and only on an intentionally-invalid request, so no account was created.</t>
+        </is>
+      </c>
+      <c r="E90" s="10" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="10" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B91" s="10" t="inlineStr">
+        <is>
+          <t>AUTO-007</t>
+        </is>
+      </c>
+      <c r="C91" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D91" s="11" t="inlineStr">
+        <is>
+          <t>Live POST to /api/auth/register with a 3-character password ('abc' for both password and confirmPassword) and email shijo-regtest-weak-20260823@mailinator.com returned HTTP 400 with body {"error":"Password must be at least 8 characters"}. The 8-character minimum is enforced server-side, not only in the client form. No account created.</t>
+        </is>
+      </c>
+      <c r="E91" s="10" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="10" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B92" s="10" t="inlineStr">
+        <is>
+          <t>AUTO-008</t>
+        </is>
+      </c>
+      <c r="C92" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D92" s="11" t="inlineStr">
+        <is>
+          <t>Fetched all 13 protected routes live with credentials:'omit' (no session cookie): /admin, /admin/terms, /admin/tickets, /admin/users, /dashboard, /dashboard/ai-visibility, /dashboard/analytics, /dashboard/billing, /dashboard/content, /dashboard/keywords, /dashboard/settings, /dashboard/tools, /dashboard/tools/keyword-research. With redirect:'manual' every one returned type 'opaqueredirect' (i.e. a real 30x, not a 200 with content); with redirect:'follow' every one resolved to /login?redirect=&lt;url-encoded original path&gt;. All 13 response bodies were byte-identical at 14,076 bytes -- the login page -- and every body was scanned for authenticated-UI markers ('Sign out', 'Usage this month', 'planTier', 'Upgrade your plan') with zero hits. No authenticated UI leaked on any route. Matches the middleware.ts matcher ['/dashboard/:path*','/admin/:path*'].</t>
+        </is>
+      </c>
+      <c r="E92" s="10" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="10" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B93" s="10" t="inlineStr">
+        <is>
+          <t>AUTO-009</t>
+        </is>
+      </c>
+      <c r="C93" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D93" s="11" t="inlineStr">
+        <is>
+          <t>Fetched all 4 endpoints live with credentials:'omit', using the correct verb for each: /api/usage GET -&gt; 401 {"error":"Not authenticated"}; /api/stripe/create-checkout POST -&gt; 401 {"error":"Please sign in first"}; /api/dashboard/ai-visibility-waitlist POST -&gt; 401 {"success":false,"error":"Please sign in to join the waitlist."}; /api/generate POST -&gt; 401 {"success":false,"error":"Please sign in to use AI tools"}. All four reject anonymous requests before doing any work. Consistent with 2026-08-22.</t>
+        </is>
+      </c>
+      <c r="E93" s="10" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="10" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B94" s="10" t="inlineStr">
+        <is>
+          <t>AUTO-010</t>
+        </is>
+      </c>
+      <c r="C94" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D94" s="11" t="inlineStr">
+        <is>
+          <t>Read app/api/stripe/create-checkout/route.ts. VALID_PLANS keys are exactly {pro, growth}. Reconciled against lib/stripe/products.ts: PLAN_FEATURES.enterprise carries comingSoon:true (paused) and free is not a paid tier, so {pro, growth} is precisely the currently-purchasable set -- no hardcoded assumption, this was derived from products.ts as the spec requires. 'enterprise' and any unrecognized plan name fall through to the 400 'Invalid plan selected' branch (lines 51-54). The interval-resolution guard is present at lines 56-62: growth has no annual priceId, so plan:'growth'+interval:'annual' correctly returns 400 'This plan is not available on that billing interval yet' rather than passing undefined to Stripe. An invalid interval value is rejected earlier at lines 40-45. The 401 auth check runs before any plan validation, independently re-verified live in AUTO-009.</t>
+        </is>
+      </c>
+      <c r="E94" s="10" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="10" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B95" s="10" t="inlineStr">
+        <is>
+          <t>AUTO-011</t>
+        </is>
+      </c>
+      <c r="C95" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D95" s="11" t="inlineStr">
+        <is>
+          <t>Fetched https://www.shijo.ai/sitemap.xml live (2,218 bytes, readable XML). 13 &lt;loc&gt; entries: /blog plus 3 blog posts, the homepage, /terms, /privacy, /cookies, /gdpr-compliance, /ai-compliance, /security, /contact, /ai-marketing-tools. Filtered all entries for /dashboard, /admin, /login and /register -- zero matches. No private or authenticated route is exposed to crawlers. Live contents match app/sitemap.ts.</t>
+        </is>
+      </c>
+      <c r="E95" s="10" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B96" s="7" t="inlineStr">
+        <is>
+          <t>AUTO-013</t>
+        </is>
+      </c>
+      <c r="C96" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="D96" s="6" t="inlineStr">
+        <is>
+          <t>Two violations, one long-standing and one NEW and previously undetected. (1) NEW -- live in public marketing copy right now: components/landing/Pricing.tsx renders '2 AI tools (Haiku-powered)' (line 27) and 'Sonnet AI for complex tasks' (lines 48 and 69) in the homepage pricing cards. Confirmed visible in the live rendered homepage body text, not just source. Haiku and Sonnet are Claude model names, so this identifies the underlying AI vendor in customer-facing marketing copy, which the product rule restricts to /privacy, /security and /ai-compliance. Every prior run missed this because the test's grep pattern is only 'claude|anthropic' -- these strings do not contain either word. It has been live since commit fcd06fa (2026-07-19 pricing restructure), i.e. roughly 35 days. Notably the repo already has the compliant wording elsewhere: components/lp/LandingPageContent.tsx says 'Advanced AI for complex tasks' and that is what /ai-marketing-tools serves live (zero haiku/sonnet matches in its HTML), so the homepage is the inconsistent surface and the fix is to copy that phrasing across. Recommend widening this test's pattern to 'claude|anthropic|haiku|sonnet|opus' for rendered JSX text going forward. (2) PERSISTS, unchanged since 2026-07-20 (now 34 days): app/gdpr-compliance/page.tsx:77 renders visible public text 'Anthropic -- AI model infrastructure powering platform features' on /gdpr-compliance, which is not one of the three approved disclosure locations. Still a policy-scope question awaiting Sri: either add /gdpr-compliance as a fourth approved location (defensible -- it is a legal/compliance page listing sub-processors, exactly the context the rule carves out) or drop the vendor name there. Unchanged non-violations (backend code and non-rendered text): app/api/generate/route.ts SDK import + model ID constants + a code comment, lib/ai/claude.ts (entire module is backend SDK plumbing), lib/tools/usage.ts:49 code comment, app/layout.tsx:14-16 code comment documenting a past fix, app/robots.ts:20 'Claude-Web' crawler allow-directive alongside GPTBot/PerplexityBot (technical SEO), and the internal 'haiku'/'sonnet' modelTier enum values in registry.ts/usage.ts/products.ts which are never rendered as-is (ToolPage.tsx:143 and dashboard/tools/page.tsx:89 correctly map them to the neutral labels 'Fast'/'Advanced'). Live homepage, /ai-marketing-tools and /contact HTML all return zero matches for 'claude' or 'anthropic'.</t>
+        </is>
+      </c>
+      <c r="E96" s="7" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="10" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B97" s="10" t="inlineStr">
+        <is>
+          <t>AUTO-015</t>
+        </is>
+      </c>
+      <c r="C97" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D97" s="11" t="inlineStr">
+        <is>
+          <t>Diffed the tool list in lib/email.ts buildWelcomeEmail() against the TOOLS export in lib/tools/registry.ts. Both contain exactly 12 tools and the sets match name-for-name with no extras or omissions (ordering differs, which is cosmetic): Post Caption Generator, Keyword Research, SEO Content Brief, SEO Meta Generator, FAQ Generator, AI Overview Optimizer, Ad Copy Generator, Ad Headline A/B Tester, Audience Targeting Profiles, Landing Page Copy Generator, Email Sequence Generator, Newsletter Generator. Also re-verified the email's free:true flags (Post Caption Generator at email.ts:34, SEO Meta Generator at email.ts:37) match exactly the two registry entries carrying minPlan:'free' (registry.ts:60 and :110), so the welcome email does not promise free access to a gated tool. No drift since the 2026-07-19 fix that removed the 24 fabricated tool names.</t>
+        </is>
+      </c>
+      <c r="E97" s="10" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B98" s="7" t="inlineStr">
+        <is>
+          <t>AUTO-016</t>
+        </is>
+      </c>
+      <c r="C98" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="D98" s="6" t="inlineStr">
+        <is>
+          <t>One item fixed, one still live. (1) FIXED since last run: the JSON-LD AggregateOffer highPrice:'99' on app/page.tsx and app/ai-marketing-tools/page.tsx -- which asserted to Google that a $99 tier was currently purchasable when Enterprise is paused -- now reads '199' in source and in the live rendered ld+json on both pages. (2) STILL FAILING, unchanged since 2026-08-22: components/landing/UseCases.tsx:24 renders 'Trusted by marketing teams, agencies, and brands worldwide' live on the homepage, under a 'Built for Modern Enterprises' heading. Confirmed present in the live homepage HTML this run. That is an unverifiable social-proof claim; lib/stripe/products.ts documents zero customers on any plan as of 2026-07-19 and the current count could not be checked this run (no Stripe MCP, no DB access), so this needs Sri to confirm real customers exist or soften the wording -- it is not safely auto-fixable. (3) Unchanged and still clean: components/landing/TrustBadges.tsx retains fabricated 'SOC 2 Compliant' / '99.9% Uptime' / '500+ Enterprises' badges but remains orphaned -- grep across app/, components/ and lib/ finds the identifier only in its own definition, zero imports, and none of that text appears in the live homepage, /ai-marketing-tools or /contact HTML fetched this run. app/layout.tsx metadata is clean (12-tool product described accurately, no certifications claimed) and app/page.tsx JSON-LD still correctly omits aggregateRating. (4) NEW, latent not live -- flagging so it does not ship by accident: lib/seo-config.ts pages.features and pages.dashboard describe unbuilt capabilities as if they exist ('keyword clustering, intent classification, search volume checking, SERP analysis, and rank tracking', 'Enterprise-grade SEO tools', 'measuring AI search visibility', 'Real-time SEO analytics' -- AI visibility is a waitlist page, not a shipped feature). The file's own comment confirms only pages.home is wired up and the rest is dead config, so nothing is currently rendered from it, but any future route that calls generatePageMetadata('features') or ('dashboard') would immediately publish fabricated feature claims. Recommend deleting the dead entries rather than leaving them as a trap.</t>
+        </is>
+      </c>
+      <c r="E98" s="7" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
GEO: fix prompt pluralisation, add identity gate and non-answer detection
First live scan scored a yoga studio 0/100 against answers about AT&T and Texas Instruments. Three causes, all fixed: (1) naive plural produced 'businesss'; (2) with Places unresolved the category fell back to a generic noun, so prompts asked about businesses in general - now returns band 'unverified' with no score instead of a confident zero; (3) four of eight replies were clarifying questions naming no business and were being counted as 'not mentioned' - now excluded from scoring, same rule as a failed request.

Adds scripts/geo-tests (151 assertions, 6 suites, real modules with fetch intercepted) and extends scripts/verify-geo-pass.sh with suite execution and an opt-in --live-scan key-health probe.
</commit_message>
<xml_diff>
--- a/docs/testing/Automated-Regression-Test-Suite.xlsx
+++ b/docs/testing/Automated-Regression-Test-Suite.xlsx
@@ -152,7 +152,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -218,6 +218,30 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1452,7 +1476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E98"/>
+  <dimension ref="A1:E141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4108,6 +4132,1167 @@
         </is>
       </c>
     </row>
+    <row r="99">
+      <c r="A99" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B99" s="27" t="inlineStr">
+        <is>
+          <t>AUTO-001</t>
+        </is>
+      </c>
+      <c r="C99" s="27" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D99" s="28" t="inlineStr">
+        <is>
+          <t>Repo: grep -rniE '24.{0,15}(tools|apps)' across app/, components/, lib/ returned exactly one hit, lib/email.ts:217, and it is a false positive -- the match is the inline CSS 'margin: 0 0 24px 0;"&gt;Tools', not a count claim. Broader sweep for any numeric tool/app count found only two numbers in use: '12' (total) and '2' (free tier). '12' is correct: lib/tools/registry.ts TOOLS has exactly 12 entries (a raw grep for 'id:' returns 14, but 2 of those are TypeScript interface field declarations at lines 20 and 29, not tools). '2' is correct per PLAN_FEATURES.free.aiToolsAccess = 2. Live: fetched raw HTML of /, /ai-marketing-tools and /contact and regex-extracted every '&lt;number&gt; tools/apps' phrase -- the complete set across all three pages is {12 tools, 12 Tools, 12 AI tools, 2 tools, 2 AI tools}. Zero occurrences of 24 or any other count. Homepage additionally renders exactly 12 tool cards, name-for-name matching the registry.</t>
+        </is>
+      </c>
+      <c r="E99" s="27" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B100" s="27" t="inlineStr">
+        <is>
+          <t>AUTO-002</t>
+        </is>
+      </c>
+      <c r="C100" s="27" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D100" s="28" t="inlineStr">
+        <is>
+          <t>Repo: grep -rn '\$99' across app/, components/, lib/ returned zero matches. Every '$29' and '$199' hit reconciles to lib/stripe/products.ts (PLAN_FEATURES.pro.price=29 displayed 'Standard', PLAN_FEATURES.growth.price=199 displayed 'Pro'). Two residual bare '99' occurrences, both benign and both already documented: (a) lib/stripe/products.ts:94-95 PLAN_FEATURES.enterprise.price=99 / annualPrice=950, explicitly commented 'kept for reference, not currently sold' and gated behind comingSoon:true, and (b) components/landing/TrustBadges.tsx:7 '99.9% Uptime', which is in an orphaned unrendered file (see AUTO-016). The JSON-LD highPrice fix from 2026-08-23 is holding: app/page.tsx:22 and app/ai-marketing-tools/page.tsx:42 both read '199' with the retired-'99' incident recorded in the adjacent comment. Live: regex-extracted every '$&lt;digits&gt;' token from the raw HTML of all three public pages. Homepage = {$0, $29, $278, $199}; /ai-marketing-tools = {$0, $29, $199}; /contact = {$29, $199}. No $99 on any surface, and Enterprise renders 'Coming Soon' with no price attached. The handful of other $-tokens ($1, $17, $14, $10, $18) were each inspected in context and are Next.js RSC flight-payload references (e.g. '\"$\",\"$1\",\"c\"', '$17:metadata'), not prices.</t>
+        </is>
+      </c>
+      <c r="E100" s="27" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="29" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B101" s="29" t="inlineStr">
+        <is>
+          <t>AUTO-003</t>
+        </is>
+      </c>
+      <c r="C101" s="29" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="D101" s="30" t="inlineStr">
+        <is>
+          <t>CRITICAL. Three defects, one long-standing and two NEW this run. (1) PERSISTS, unchanged since first logged 2026-08-22 (now 3rd consecutive run): app/api/stripe/create-checkout/route.ts:81 returns `You are already on the ${plan} plan` interpolating the RAW internal key; app/dashboard/billing/page.tsx:143 does setError(data.error) and line 216 renders {error} verbatim into the visible red banner. A $199 customer who re-clicks upgrade is shown 'You are already on the growth plan'. One-line fix: PLAN_DISPLAY_NAME[plan]. (2) NEW, previously undetected, and it reaches EVERY new signup: lib/email.ts buildWelcomeEmail() line 172 badges every non-free tool with the literal string 'Pro' -- but all 12 tools unlock on the $29 tier, which is displayed as 'Standard'; 'Pro' is the $199 tier. The same email's upgrade CTA 50 lines later (line 223) reads 'Unlock all 12 tools for just $29/month'. So the welcome email labels a tool 'Pro' and then prices it at Standard's price in the same message. Correct badge text is 'Standard'. (3) NEW, previously undetected, live in product UI: components/dashboard/TopBar.tsx:11 rotating tip reads 'Pro gives you 200/month across all 12 tools.' 200 gens/month is Standard; Pro is 1,500 (PLAN_FEATURES.growth.aiToolsMonthly=1500). The tip both names the wrong plan and understates Pro by 7.5x. Clean elsewhere: no raw {userPlan}/{planTier} interpolation anywhere in app/ or components/; PLAN_DISPLAY_NAME correctly imported and used by admin/users, dashboard/billing (x3), dashboard/page, dashboard/settings, Sidebar and UsageMeter. Live public HTML plan names extracted as exactly {Free, Standard, Pro, Enterprise} on all three pages, zero raw 'growth' leaks. Dashboard billing HTML still not diffable unauthenticated -- it correctly 30x-redirects to /login -- so (1),(2),(3) are verified at code level only.</t>
+        </is>
+      </c>
+      <c r="E101" s="29" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B102" s="27" t="inlineStr">
+        <is>
+          <t>AUTO-004</t>
+        </is>
+      </c>
+      <c r="C102" s="27" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D102" s="28" t="inlineStr">
+        <is>
+          <t>Pass. RESOLVED after 4 blocked runs. Still no Stripe MCP connector (list_connectors returns []), so this was run by reading the LIVE Stripe dashboard directly in a connected Chrome session (account acct_1Sr24rHTpiuftGGE, live mode, read-only -- nothing was edited). All three Products referenced by STRIPE_PRICE_IDS check out against PLAN_DISPLAY_NAME: prod_UAltLAeJGLVSqI ($29, price_1TCQLpHTpiuftGGEZWt9UJ2Y) name = 'SHIJO.AI Standard' -- correct, metadata tier='pro', description 'All 12 AI marketing tools, 200 generations/month, advanced AI models.' The 2026-07-19 'Shijo Pro' mislabel is confirmed fixed and the fix is documented in the product's own internal_note metadata. prod_UuvJvC2ZKysgfK ($199, price_1Tv5SpHTpiuftGGEMu4TdOzs) name = 'SHIJO.AI Pro' -- correct, metadata tier='growth', description '...1,500 generations/month...'. prod_UAluQCvL32SQ3k (Enterprise, paused) name = 'SHIJO.AI Enterprise' -- correct, metadata status='paused'. SUB-FINDING, new and not previously logged -- stale PRICE nicknames (distinct from Product names, which is what this test asserts, hence Pass not Fail): the $278/yr price under the Standard product is still nicknamed 'Shijo Pro Annual' (created 7/17/26), and the Enterprise annual price is 'Shijo Enterprise Annual'. Both carry the retired 'Shijo Pro' branding the product names were renamed away from on 2026-07-19 -- the rename covered Products but never the Prices. Severity is low because Stripe price nicknames are internal-dashboard-only and do not render on Checkout (the Product name and description do, and both are correct), but price_1TuEaIHTpiuftGGEslehCB4Y IS purchasable via VALID_PLANS.pro.annual, so this is live drift of the same class this test exists to catch. Recommend renaming to 'SHIJO.AI Standard Annual'. ALSO MATERIAL, affects AUTO-016: the Standard product now shows MRR $29.00 and 1 active subscription. The 'zero customers on any plan' baseline recorded in lib/stripe/products.ts (2026-07-19) is out of date -- there is now 1 paying customer. That still does not substantiate the homepage's 'Trusted by marketing teams, agencies, and brands worldwide' (plural, worldwide), so AUTO-016 finding (1) stands.</t>
+        </is>
+      </c>
+      <c r="E102" s="27" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B103" s="27" t="inlineStr">
+        <is>
+          <t>AUTO-005</t>
+        </is>
+      </c>
+      <c r="C103" s="27" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D103" s="28" t="inlineStr">
+        <is>
+          <t>Live POST to https://www.shijo.ai/api/auth/register with email 'not-a-valid-email' (name 'Regression Bot', matching valid 8+ char passwords so email format was the only invalid field) -&gt; HTTP 400, body {"error":"Please enter a valid email address"}. Not 200; no account created. Method note: the sandbox egress proxy blocks www.shijo.ai (CONNECT returns 403 X-Proxy-Error: blocked-by-allowlist), so curl was unavailable this run; the request was issued as a same-origin fetch with credentials:'omit' from a connected Chrome session on www.shijo.ai, which exercises the identical live endpoint and is the same method used on 2026-08-23.</t>
+        </is>
+      </c>
+      <c r="E103" s="27" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B104" s="27" t="inlineStr">
+        <is>
+          <t>AUTO-006</t>
+        </is>
+      </c>
+      <c r="C104" s="27" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D104" s="28" t="inlineStr">
+        <is>
+          <t>Live POST to /api/auth/register with password 'ValidPass123!' and confirmPassword 'DifferentPass456!' (throwaway address shijo-regress-20260824a@mailinator.com) -&gt; HTTP 400, body {"error":"Passwords do not match"}. The server-side confirmPassword check shipped 2026-07-19 is still live. No account created. Same same-origin-fetch method as AUTO-005 (sandbox curl blocked by proxy allowlist).</t>
+        </is>
+      </c>
+      <c r="E104" s="27" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B105" s="27" t="inlineStr">
+        <is>
+          <t>AUTO-007</t>
+        </is>
+      </c>
+      <c r="C105" s="27" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D105" s="28" t="inlineStr">
+        <is>
+          <t>Live POST to /api/auth/register with a 3-character password 'abc' in both password and confirmPassword (throwaway address shijo-regress-20260824b@mailinator.com) -&gt; HTTP 400, body {"error":"Password must be at least 8 characters"}. The 8-character minimum is enforced server-side, independent of the client form. No account created. Same same-origin-fetch method as AUTO-005.</t>
+        </is>
+      </c>
+      <c r="E105" s="27" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B106" s="27" t="inlineStr">
+        <is>
+          <t>AUTO-008</t>
+        </is>
+      </c>
+      <c r="C106" s="27" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D106" s="28" t="inlineStr">
+        <is>
+          <t>Fetched all 15 protected routes live with credentials:'omit' (no session cookie), redirect:'follow', and asserted the final URL matched /login?redirect=. 15/15 passed. Routes covered -- dashboard: /dashboard, /dashboard/ai-visibility, /dashboard/analytics, /dashboard/billing, /dashboard/content, /dashboard/keywords, /dashboard/settings, /dashboard/tools, /dashboard/tools/keyword-research (dynamic [toolId] segment); admin: /admin, /admin/signups, /admin/terms, /admin/tickets, /admin/usage, /admin/users. Route list was re-derived this run from `find app/dashboard app/admin -name page.tsx` rather than reused, so newly added pages are covered. Every one landed on https://www.shijo.ai/login?redirect=&lt;url-encoded original path&gt; -- i.e. a real redirect, with the return path preserved, not a 200 carrying authenticated UI. Matches middleware.ts, whose matcher is ['/dashboard/:path*','/admin/:path*'] and which redirects to /login when the session cookie is absent or the JWT payload fails to decode/is expired.</t>
+        </is>
+      </c>
+      <c r="E106" s="27" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B107" s="27" t="inlineStr">
+        <is>
+          <t>AUTO-009</t>
+        </is>
+      </c>
+      <c r="C107" s="27" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D107" s="28" t="inlineStr">
+        <is>
+          <t>Fetched all 4 endpoints live with credentials:'omit', probing BOTH GET and POST on each to make sure nothing leaks on the unintended verb. On their real method all four return 401: /api/usage GET -&gt; 401 {"error":"Not authenticated"}; /api/stripe/create-checkout POST -&gt; 401 {"error":"Please sign in first"}; /api/dashboard/ai-visibility-waitlist POST -&gt; 401 {"success":false,"error":"Please sign in to join the waitlist."}; /api/generate POST -&gt; 401 {"success":false,"error":"Please sign in to use AI tools"}. On the wrong verb the POST-only routes return 405 with an empty body (/api/stripe/create-checkout GET, /api/dashboard/ai-visibility-waitlist GET, /api/generate GET) and /api/usage POST returns 405 empty. No endpoint returned data, and no error body disclosed anything beyond the sign-in prompt.</t>
+        </is>
+      </c>
+      <c r="E107" s="27" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B108" s="27" t="inlineStr">
+        <is>
+          <t>AUTO-010</t>
+        </is>
+      </c>
+      <c r="C108" s="27" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D108" s="28" t="inlineStr">
+        <is>
+          <t>Read app/api/stripe/create-checkout/route.ts. VALID_PLANS keys are exactly {pro, growth} -- 'enterprise' is absent, with an explanatory comment recording that it was paused on 2026-07-19. Cross-checked against lib/stripe/products.ts rather than hardcoding: PLAN_FEATURES.enterprise carries comingSoon:true and free has no priceId, so {pro, growth} is precisely the currently-purchasable set. Both guards are present and correct: `if (!plan || !VALID_PLANS[plan])` -&gt; 400 'Invalid plan selected' catches 'enterprise' and any unrecognized name, and the interval-resolution guard `if (!VALID_PLANS[plan][interval])` -&gt; 400 'This plan is not available on that billing interval yet' correctly handles growth having monthly but no annual price. A preceding check rejects any interval other than monthly/annual with 400. Server-side enforcement holds regardless of what the pricing UI shows.</t>
+        </is>
+      </c>
+      <c r="E108" s="27" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B109" s="27" t="inlineStr">
+        <is>
+          <t>AUTO-011</t>
+        </is>
+      </c>
+      <c r="C109" s="27" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D109" s="28" t="inlineStr">
+        <is>
+          <t>Fetched https://www.shijo.ai/sitemap.xml live. 13 &lt;loc&gt; entries, all public: /, /blog plus 3 blog posts (ai-seo-tools-keyword-research-faster, ai-ad-copy-that-converts, ai-marketing-tools-small-business-2026), /ai-marketing-tools, /contact, and the 6 legal pages (/terms, /privacy, /cookies, /gdpr-compliance, /ai-compliance, /security). Zero matches for 'dashboard' or 'admin'. Count is up from 12 on 2026-08-23 because the /blog index is now included alongside the 3 posts -- an intended addition, not a leak. Consistent with AUTO-008: the same routes that redirect to /login are also absent from the crawlable sitemap.</t>
+        </is>
+      </c>
+      <c r="E109" s="27" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="29" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B110" s="29" t="inlineStr">
+        <is>
+          <t>AUTO-013</t>
+        </is>
+      </c>
+      <c r="C110" s="29" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="D110" s="30" t="inlineStr">
+        <is>
+          <t>Both violations from 2026-08-23 persist unchanged; nothing new. (1) STILL LIVE in public marketing copy, now 41 days old (since commit fcd06fa, 2026-07-19): components/landing/Pricing.tsx renders '2 AI tools (Haiku-powered)' (line 27) and 'Sonnet AI for complex tasks' (lines 48 and 69) in the homepage pricing cards. Re-confirmed in the live homepage HTML this run -- a regex sweep for /claude|anthropic|haiku|sonnet|opus/i over the raw HTML of all three public pages returns {Haiku, Sonnet} on / and NOTHING on /ai-marketing-tools or /contact. Haiku and Sonnet are Claude model names, so the homepage identifies the AI vendor in customer-facing copy, which the product rule limits to /privacy, /security and /ai-compliance. The compliant wording already exists in the repo: components/lp/LandingPageContent.tsx says 'Advanced AI for complex tasks', which is exactly what /ai-marketing-tools serves live -- the fix is to copy that phrasing into Pricing.tsx lines 27/48/69. Note the test's own grep pattern ('claude|anthropic') cannot catch this; recommend the sheet's Method be widened to 'claude|anthropic|haiku|sonnet|opus'. (2) PERSISTS, unchanged since 2026-07-20 (now 40 days): app/gdpr-compliance/page.tsx:77 renders public text 'Anthropic -- AI model infrastructure powering platform features'. This remains a policy-scope question for Sri, not a code bug: either formally add /gdpr-compliance as a fourth approved disclosure location (defensible -- it is a legal page listing sub-processors, precisely the carve-out the rule intends) or drop the vendor name there. Unchanged non-violations (backend or non-rendered): app/api/generate/route.ts SDK import + model-ID constants + one comment, lib/ai/claude.ts (entire module is backend SDK plumbing), lib/tools/usage.ts:50 comment, app/layout.tsx:14-16 comment documenting the 2026-07-18 fix, app/robots.ts:20 'Claude-Web' crawler allow-directive, and the internal 'haiku'/'sonnet' modelTier enum values, which ToolPage.tsx:153 and dashboard/tools/page.tsx:89 correctly map to the neutral labels 'Fast'/'Advanced'.</t>
+        </is>
+      </c>
+      <c r="E110" s="29" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B111" s="27" t="inlineStr">
+        <is>
+          <t>AUTO-015</t>
+        </is>
+      </c>
+      <c r="C111" s="27" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D111" s="28" t="inlineStr">
+        <is>
+          <t>Diffed the tool list in lib/email.ts buildWelcomeEmail() against the TOOLS export in lib/tools/registry.ts programmatically (regex-extracted both name sets, compared as sets in both directions). 12 names each side; set difference empty both ways; exact name-for-name match: Post Caption Generator, Keyword Research, SEO Content Brief, SEO Meta Generator, FAQ Generator, AI Overview Optimizer, Ad Copy Generator, Ad Headline A/B Tester, Audience Targeting Profiles, Landing Page Copy Generator, Email Sequence Generator, Newsletter Generator. The 24-fabricated-name regression fixed on 2026-07-19 has not returned, and the hand-sync warning comment at lib/email.ts:135-139 is still in place. Free/paid split is also correct -- the two tools badged FREE (Post Caption Generator, SEO Meta Generator) are exactly the two registry entries with minPlan:'free'. NOTE: the paid-tool badge TEXT in this same email is wrong ('Pro' where it should read 'Standard') -- that is a plan-naming defect logged under AUTO-003 this run, not a tool-list mismatch, so it does not affect this result.</t>
+        </is>
+      </c>
+      <c r="E111" s="27" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="29" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B112" s="29" t="inlineStr">
+        <is>
+          <t>AUTO-016</t>
+        </is>
+      </c>
+      <c r="C112" s="29" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="D112" s="30" t="inlineStr">
+        <is>
+          <t>One item still live, two latent, one confirmed still dormant. (1) STILL FAILING, unchanged since 2026-08-22 (3rd consecutive run): components/landing/UseCases.tsx:24 renders 'Trusted by marketing teams, agencies, and brands worldwide' live on the homepage under a 'Built for Modern Enterprises' heading -- re-confirmed by regex over the live homepage HTML this run. Unverifiable social-proof claim; lib/stripe/products.ts documents zero customers on any plan as of 2026-07-19 and the current count could not be checked this run (no Stripe MCP, no DB access). Needs Sri to either confirm real customers exist or soften the wording -- not safely auto-fixable. (2) LATENT, unchanged: lib/seo-config.ts pages.features (lines 38-41) and pages.dashboard (lines 50-52) still describe unbuilt capabilities as shipped -- 'clustering, intent classification, search volume checking, SERP analysis, and rank tracking', 'Enterprise-grade SEO tools', 'measuring AI search visibility', 'Real-time SEO analytics'. AI visibility is a waitlist page, not a feature. Only pages.home is wired up, so nothing renders from these today, but any future generatePageMetadata('features'/'dashboard') call publishes fabricated claims instantly. Recommend deleting the dead entries rather than leaving the trap. (3) STILL DORMANT, unchanged: components/landing/TrustBadges.tsx retains 'SOC 2 Compliant', '99.9% Uptime', '10M+ Keywords Analyzed Daily', '500+ Enterprises'. grep across app/, components/, lib/ finds the identifier only in its own definition -- zero imports -- and a live regex sweep for /SOC ?2|99\.9%|10M\+|500\+ Enterprises/i over all three public pages returns nothing. Still needs a user-run `rm` (sandbox cannot delete). (4) CLEAN: app/layout.tsx metadata describes the real 12-tool product and claims no certifications; app/page.tsx JSON-LD correctly omits aggregateRating and reports offerCount 3 / highPrice 199.</t>
+        </is>
+      </c>
+      <c r="E112" s="29" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B113" s="27" t="inlineStr">
+        <is>
+          <t>AUTO-012</t>
+        </is>
+      </c>
+      <c r="C113" s="27" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D113" s="28" t="inlineStr">
+        <is>
+          <t>Pass. FIRST TIME THIS TEST HAS EVER RUN -- it is marked Chrome-required and every scheduled run skips it; it only ran because Sri opened a browser session after the unattended run finished, so it is logged as Ad-hoc rather than Scheduled. Loaded all four public pages in a connected Chrome tab with console capture enabled BEFORE each load (the extension only records from the point the reader is first attached, so each page was navigated fresh after enabling, not read from a pre-existing load): / , /ai-marketing-tools, /contact, /blog. Zero console errors and zero uncaught exceptions on all four, filtering onlyErrors with a 30-message limit. Note on confidence: this covers load-time errors on the four public routes only. It does NOT cover interaction-triggered errors (form submits, the contact-form captcha, pricing toggles) or any authenticated route, so it is a narrower signal than a clean bill of health for the front end.</t>
+        </is>
+      </c>
+      <c r="E113" s="27" t="inlineStr">
+        <is>
+          <t>Ad-hoc-Claude</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="10" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B114" s="10" t="inlineStr">
+        <is>
+          <t>AUTO-001</t>
+        </is>
+      </c>
+      <c r="C114" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D114" s="11" t="inlineStr">
+        <is>
+          <t>Repo: grep -rniE '24[^0-9]{0,15}(tools|apps)' across app/, components/, lib/ returned ZERO matches (the lib/email.ts:217 'margin: 0 0 24px 0' false positive that earlier runs reported does not match this tightened pattern). Broader sweep for any '&lt;number&gt; tools/apps' phrase across source found only two numbers in use, 12 and 2, both correct: lib/tools/registry.ts TOOLS has exactly 12 entries (verified programmatically by extracting the name: fields, not by counting 'id:'), and PLAN_FEATURES.free.aiToolsAccess = 2. Live: fetched the rendered HTML of /, /ai-marketing-tools and /contact. Complete set of count phrases across all three = {12 AI-Powered Marketing Tools, 12 Tools One Platform, All 12 AI tools, 12 Tools Across 4 Categories, 12 tools, 2 AI tools, 2 tools free forever}. Zero occurrences of 24 or any other count. Homepage renders exactly 12 tool cards and their names match the registry one-for-one. RUN CONTEXT: this is the SECOND scheduled run logged under 2026-08-29 -- a full 14-row scheduled set already exists for this date from an earlier fire today. Prior history was preserved, not overwritten.</t>
+        </is>
+      </c>
+      <c r="E114" s="10" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="10" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B115" s="10" t="inlineStr">
+        <is>
+          <t>AUTO-002</t>
+        </is>
+      </c>
+      <c r="C115" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D115" s="11" t="inlineStr">
+        <is>
+          <t>Repo: grep -rn '\$99' across app/, components/, lib/ returned zero matches. Every '$29' and '$199' occurrence reconciles to lib/stripe/products.ts (PLAN_FEATURES.pro.price=29 displayed 'Standard'; PLAN_FEATURES.growth.price=199 displayed 'Pro'). Two known-benign bare 99s unchanged: PLAN_FEATURES.enterprise.price=99 (commented 'kept for reference, not currently sold', gated by comingSoon:true) and TrustBadges.tsx '99.9% Uptime' in an orphaned unrendered file (see AUTO-016). Live: homepage pricing renders $0 / $29 (or $278/year, save 20%) / $199 / Enterprise 'Coming Soon' with no price; /ai-marketing-tools renders $0 / $29 / $199 / Coming Soon; /contact sidebar renders 'Standard: $29/mo' and 'Pro: $199/mo'. No $99 on any public surface. Three numbers consistent across all three pages.</t>
+        </is>
+      </c>
+      <c r="E115" s="10" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B116" s="14" t="inlineStr">
+        <is>
+          <t>AUTO-003</t>
+        </is>
+      </c>
+      <c r="C116" s="14" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="D116" s="15" t="inlineStr">
+        <is>
+          <t>CRITICAL. All three defects first logged on the earlier 2026-08-29 run are UNCHANGED -- nothing was fixed between the two runs today, and nothing new appeared. (1) app/api/stripe/create-checkout/route.ts:81 returns `You are already on the ${plan} plan` interpolating the RAW internal key; app/dashboard/billing/page.tsx:143 does setError(data.error) and line 216 renders {error} verbatim in the visible red banner -- a $199 customer re-clicking upgrade sees 'You are already on the growth plan'. Fix: PLAN_DISPLAY_NAME[plan]. First logged 2026-08-22, now 4 consecutive runs. (2) lib/email.ts buildWelcomeEmail() line ~171 badges every non-free tool with the literal string 'Pro', but all 12 tools unlock on the $29 tier displayed as 'Standard'; the same email's CTA at line 223 reads 'Unlock all 12 tools for just $29/month'. The email labels a tool 'Pro' then prices it at Standard's price. Reaches every new signup. Correct badge text is 'Standard'. (3) components/dashboard/TopBar.tsx:11 rotating tip reads 'Pro gives you 200/month across all 12 tools' -- 200/mo is Standard; Pro is 1,500 (PLAN_FEATURES.growth.aiToolsMonthly=1500). Wrong plan name AND understates Pro by 7.5x. Clean elsewhere: the only ${plan}/{userPlan}/{planTier} interpolations in app/ or components/ are the one in (1) plus a success_url query param (harmless); PLAN_DISPLAY_NAME is correctly imported and used in admin/users, dashboard/billing (x3), dashboard/page, dashboard/settings, Sidebar and UsageMeter. Live public HTML plan names on all three pages are exactly {Free, Standard, Pro, Enterprise} with zero raw 'growth' leaks. The dashboard billing page could not be diffed -- it correctly redirects unauthenticated -- so (1),(2),(3) are code-level verification only.</t>
+        </is>
+      </c>
+      <c r="E116" s="14" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="16" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B117" s="16" t="inlineStr">
+        <is>
+          <t>AUTO-004</t>
+        </is>
+      </c>
+      <c r="C117" s="16" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="D117" s="17" t="inlineStr">
+        <is>
+          <t>BLOCKED -- and this is a Critical-priority test. No Stripe MCP connector is available in this session (a ToolSearch for stripe/payments/products/prices returns no deferred tools, and the connector registry exposes none). The fallback the earlier 2026-08-29 run used -- reading the live Stripe dashboard in a connected Chrome session -- is also unavailable: mcp__claude-in-chrome__list_connected_browsers returns [], and the built-in browser pane refuses www.shijo.ai and by extension any external navigation, so there is no way to reach dashboard.stripe.com unattended. Nothing was verified against Stripe this run. The three Products that need checking are unchanged in the repo: prod_UAltLAeJGLVSqI (price_1TCQLpHTpiuftGGEZWt9UJ2Y, $29, must read 'SHIJO.AI Standard'), prod_UuvJvC2ZKysgfK (price_1Tv5SpHTpiuftGGEMu4TdOzs, $199, must read 'SHIJO.AI Pro'), prod_UAluQCvL32SQ3k (Enterprise, paused). Carrying forward from the earlier run today, still OPEN and unverified this run: the $278/yr price under the Standard product is still nicknamed 'Shijo Pro Annual' and the Enterprise annual price 'Shijo Enterprise Annual' -- retired branding on a price that IS purchasable via VALID_PLANS.pro.annual. To unblock permanently, connect a Stripe MCP connector; that is the only way this Critical test runs on a truly unattended schedule.</t>
+        </is>
+      </c>
+      <c r="E117" s="16" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="16" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B118" s="16" t="inlineStr">
+        <is>
+          <t>AUTO-005</t>
+        </is>
+      </c>
+      <c r="C118" s="16" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="D118" s="17" t="inlineStr">
+        <is>
+          <t>BLOCKED -- no way to issue a POST to the live site this run. Three transports were tried and all failed: (a) sandbox curl -- the egress proxy rejects www.shijo.ai at CONNECT with HTTP 403 and header X-Proxy-Error: blocked-by-allowlist; (b) built-in browser pane -- navigate to https://www.shijo.ai/ returns 'navigation to https://shijo.ai was denied or failed', retried three times including with force:true, so the same-origin-fetch method used on 2026-08-23 and earlier today is unavailable; (c) Chrome extension -- list_connected_browsers returns [], no browser attached. mcp__workspace__web_fetch works for public GETs but cannot send POST bodies or surface status codes. No request was sent to /api/auth/register, so no account was created and nothing about the invalid-email validation was verified this run. Last known good: Pass earlier today (400 'Please enter a valid email address').</t>
+        </is>
+      </c>
+      <c r="E118" s="16" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="16" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B119" s="16" t="inlineStr">
+        <is>
+          <t>AUTO-006</t>
+        </is>
+      </c>
+      <c r="C119" s="16" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="D119" s="17" t="inlineStr">
+        <is>
+          <t>BLOCKED -- same transport failure as AUTO-005 (sandbox curl blocked by proxy allowlist, built-in browser denies www.shijo.ai, Chrome extension not connected, web_fetch is GET-only). No POST was sent to /api/auth/register, so the server-side password/confirmPassword mismatch check shipped 2026-07-19 was NOT exercised this run. No account created. Last known good: Pass earlier today (400 'Passwords do not match').</t>
+        </is>
+      </c>
+      <c r="E119" s="16" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="16" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B120" s="16" t="inlineStr">
+        <is>
+          <t>AUTO-007</t>
+        </is>
+      </c>
+      <c r="C120" s="16" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="D120" s="17" t="inlineStr">
+        <is>
+          <t>BLOCKED -- same transport failure as AUTO-005/006. The 8-character server-side minimum was not exercised this run; no POST reached /api/auth/register and no account was created. Last known good: Pass earlier today (400 'Password must be at least 8 characters').</t>
+        </is>
+      </c>
+      <c r="E120" s="16" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="16" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B121" s="16" t="inlineStr">
+        <is>
+          <t>AUTO-008</t>
+        </is>
+      </c>
+      <c r="C121" s="16" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="D121" s="17" t="inlineStr">
+        <is>
+          <t>BLOCKED (partial evidence only). web_fetch enforces a provenance rule -- it will only retrieve URLs that appeared in a prior fetch result or a user message -- so only routes linked from public pages were reachable. Of the 15 protected routes, exactly one was fully verified live: GET https://www.shijo.ai/dashboard (linked from the site footer) followed a redirect to https://www.shijo.ai/login?redirect=%2Fdashboard and rendered the Sign In page with meta-robots noindex -- correct behaviour, no authenticated UI leaked. /dashboard/billing (linked from /contact) returned an empty body with no status code exposed -- inconclusive. All /admin/* routes were rejected outright with 'URL not in provenance set' and were not tested at all. No POST/status-code transport was available (see AUTO-005). Code-level cross-check DID pass and is the reason this is Blocked rather than Fail: middleware.ts has matcher ['/dashboard/:path*','/admin/:path*'] and redirects to /login?redirect=&lt;pathname&gt; whenever the session cookie is absent or decodeJWTPayload returns null (bad shape, missing userId/email, or expired exp). Route inventory re-derived this run via find: 14 page.tsx files across app/dashboard and app/admin -- note app/admin/page.tsx does NOT exist, so the '15 routes' figure in earlier logs counted a bare /admin index that is not a page (it is still covered by the matcher). Full live sweep needs a connected browser.</t>
+        </is>
+      </c>
+      <c r="E121" s="16" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="16" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B122" s="16" t="inlineStr">
+        <is>
+          <t>AUTO-009</t>
+        </is>
+      </c>
+      <c r="C122" s="16" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="D122" s="17" t="inlineStr">
+        <is>
+          <t>BLOCKED -- the four endpoints (/api/usage, /api/stripe/create-checkout, /api/dashboard/ai-visibility-waitlist, /api/generate) could not be probed. Sandbox curl is blocked by the egress proxy allowlist, the built-in browser pane refuses www.shijo.ai, and no Chrome extension is connected; web_fetch cannot POST and does not surface HTTP status codes, so it cannot distinguish a 401 from a 200. Zero endpoints verified this run. Partial code-level reassurance only, not a substitute for the live check: app/api/stripe/create-checkout/route.ts was read in full for AUTO-010 and its first statement after the try is a getSession() null-check returning 401 'Please sign in first' before any body parsing or DB access. The other three routes were not read. Last known good: Pass earlier today, all four 401 on their real verb and 405 on the wrong verb.</t>
+        </is>
+      </c>
+      <c r="E122" s="16" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="10" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B123" s="10" t="inlineStr">
+        <is>
+          <t>AUTO-010</t>
+        </is>
+      </c>
+      <c r="C123" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D123" s="11" t="inlineStr">
+        <is>
+          <t>Read app/api/stripe/create-checkout/route.ts in full. VALID_PLANS keys are exactly {pro, growth}; 'enterprise' is absent with an inline comment recording the 2026-07-19 pause. Cross-checked against lib/stripe/products.ts rather than hardcoding the expected set: PLAN_FEATURES.enterprise carries comingSoon:true and PLAN_FEATURES.free has no priceId, so {pro, growth} is exactly the currently-purchasable set. Three guards present and correct: interval must be 'monthly' or 'annual' (else 400 'Invalid billing interval'); !plan || !VALID_PLANS[plan] -&gt; 400 'Invalid plan selected', which catches 'enterprise' and every unrecognized name; and the interval-resolution guard !VALID_PLANS[plan][interval] -&gt; 400 'This plan is not available on that billing interval yet', which correctly handles growth having monthly but no annual price. Also re-verified the sibling route app/api/billing/checkout/route.ts, since it can reach Stripe too: its ALLOWED_PRICE_IDS is a hand-written list of exactly PRO_MONTHLY, PRO_ANNUAL, GROWTH_MONTHLY -- deliberately not Object.values(STRIPE_PRICE_IDS), so the paused ENTERPRISE_* and sandbox CREDITS_* ids are not purchasable there either. Server-side enforcement holds independently of the pricing UI.</t>
+        </is>
+      </c>
+      <c r="E123" s="10" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="10" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B124" s="10" t="inlineStr">
+        <is>
+          <t>AUTO-011</t>
+        </is>
+      </c>
+      <c r="C124" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D124" s="11" t="inlineStr">
+        <is>
+          <t>Fetched https://www.shijo.ai/sitemap.xml live. 13 &lt;loc&gt; entries, zero matches for 'dashboard' or 'admin'. Full list: /blog, 3 blog posts (ai-seo-tools-keyword-research-faster, ai-ad-copy-that-converts, ai-marketing-tools-small-business-2026), the root, and the 6 legal pages (/terms, /privacy, /cookies, /gdpr-compliance, /ai-compliance, /security), plus /contact and /ai-marketing-tools. Identical to the earlier run today. Consistent with AUTO-008: the routes middleware.ts redirects to /login are also absent from the crawlable sitemap, so there is no information-disclosure path via search.</t>
+        </is>
+      </c>
+      <c r="E124" s="10" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B125" s="14" t="inlineStr">
+        <is>
+          <t>AUTO-013</t>
+        </is>
+      </c>
+      <c r="C125" s="14" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="D125" s="15" t="inlineStr">
+        <is>
+          <t>Both violations persist unchanged; nothing new, nothing fixed since the earlier run today. (1) STILL LIVE in public marketing copy, now 41 days old: components/landing/Pricing.tsx renders '2 AI tools (Haiku-powered)' (line 27) and 'Sonnet AI for complex tasks' (lines 48 and 69). Re-confirmed in the live homepage HTML this run -- the Free card reads '2 AI tools (Haiku-powered)' and both the Standard and Pro cards read 'Sonnet AI for complex tasks'. Haiku and Sonnet are Claude model names, so the homepage identifies the AI vendor in customer-facing copy, which the product rule confines to /privacy, /security and /ai-compliance. /ai-marketing-tools and /contact are clean -- /ai-marketing-tools serves the already-compliant wording 'Advanced AI for complex tasks' from components/lp/LandingPageContent.tsx, which is exactly the string to copy into Pricing.tsx lines 27/48/69. The sheet's own grep pattern ('claude|anthropic') cannot catch this; recommend widening the Method to 'claude|anthropic|haiku|sonnet|opus'. (2) PERSISTS, unchanged since 2026-07-20: app/gdpr-compliance/page.tsx:77 renders public text 'Anthropic -- AI model infrastructure powering platform features'. Still a policy-scope decision for Sri, not a code bug -- either formally add /gdpr-compliance as a fourth approved disclosure location (defensible: it is a legal page listing sub-processors, exactly the carve-out the rule intends, and it is in the sitemap alongside the three approved pages) or drop the vendor name. Confirmed non-violations (backend or non-rendered, unchanged): app/api/generate/route.ts SDK import + model-id constants + one code comment, app/layout.tsx:14-16 comment documenting the 2026-07-18 fix, app/robots.ts:20 'Claude-Web' crawler allow-directive, and the internal haiku/sonnet modelTier enum values that ToolPage.tsx and dashboard/tools map to the neutral labels Fast/Advanced.</t>
+        </is>
+      </c>
+      <c r="E125" s="14" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="10" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B126" s="10" t="inlineStr">
+        <is>
+          <t>AUTO-015</t>
+        </is>
+      </c>
+      <c r="C126" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D126" s="11" t="inlineStr">
+        <is>
+          <t>Diffed programmatically: regex-extracted the tool names from buildWelcomeEmail() in lib/email.ts and from the TOOLS export in lib/tools/registry.ts, compared as sets in both directions. 12 names each side, symmetric difference empty. Exact match: Post Caption Generator, Keyword Research, SEO Content Brief, SEO Meta Generator, FAQ Generator, AI Overview Optimizer, Ad Copy Generator, Ad Headline A/B Tester, Audience Targeting Profiles, Landing Page Copy Generator, Email Sequence Generator, Newsletter Generator. (Order differs -- the email groups by category -- which is expected and not a mismatch.) The 24-fabricated-name regression fixed 2026-07-19 has not returned, and the hand-sync warning comment at lib/email.ts:135-139 is still in place. NOTE: the paid-tool badge TEXT in this same email is wrong ('Pro' where it should read 'Standard'); that is a plan-naming defect logged under AUTO-003, not a tool-list mismatch, so it does not change this result.</t>
+        </is>
+      </c>
+      <c r="E126" s="10" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B127" s="14" t="inlineStr">
+        <is>
+          <t>AUTO-016</t>
+        </is>
+      </c>
+      <c r="C127" s="14" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="D127" s="15" t="inlineStr">
+        <is>
+          <t>One item live, two latent, one dormant -- all unchanged from the earlier run today. (1) STILL FAILING, 4th consecutive run since 2026-08-22: components/landing/UseCases.tsx:24 renders 'Trusted by marketing teams, agencies, and brands worldwide' under a 'Built for Modern Enterprises' heading, re-confirmed verbatim in the live homepage HTML this run. Unverifiable social-proof claim -- plural teams, agencies and brands, worldwide. The customer count could not be checked this run (no Stripe MCP, no DB access, see AUTO-004); the last actual reading, from the earlier run today, was 1 active subscription on Standard, which does not substantiate the wording. Needs Sri to either soften the copy or confirm real customers -- not safely auto-fixable. (2) LATENT, unchanged: lib/seo-config.ts pages.features (lines 38-41) and pages.dashboard (lines 50-52) describe unbuilt capabilities as shipped -- 'clustering, intent classification, search volume checking, SERP analysis, and rank tracking', 'Enterprise-grade SEO tools', 'tracking keywords, monitoring rankings, analyzing SERP performance, and measuring AI search visibility', 'Real-time SEO analytics'. AI visibility is a waitlist page, not a feature. The file's own comment says these are 'left in place but not linked from any route', so nothing renders today -- but any future generatePageMetadata('features'/'dashboard') call publishes fabricated claims instantly. Recommend deleting the dead entries rather than leaving the trap. (3) STILL DORMANT: components/landing/TrustBadges.tsx retains 'SOC 2 Compliant', '99.9% Uptime', '10M+ Keywords Analyzed Daily', '500+ Enterprises'. grep across app/ and components/ finds the identifier only in its own definition file -- zero imports -- and none of the four strings appear in the live HTML of any of the three public pages. Still needs a user-run rm; the sandbox cannot delete. (4) CLEAN: app/layout.tsx metadata describes the real 12-tool product and claims no certifications or awards; a sweep for SOC 2 / ISO 27001 / HIPAA / certified / award / guarantee / '&lt;N&gt;+ customers' language across layout.tsx, seo-config.ts, app/page.tsx and the landing+lp component trees surfaced nothing beyond items (1) and (3).</t>
+        </is>
+      </c>
+      <c r="E127" s="14" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="31" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B128" s="31" t="inlineStr">
+        <is>
+          <t>AUTO-001</t>
+        </is>
+      </c>
+      <c r="C128" s="31" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D128" s="22" t="inlineStr">
+        <is>
+          <t>Repo: grep -rniE '24[^0-9]{0,15}(tools|apps)' across app/, components/, lib/ returned ZERO matches. Broader sweep for any '&lt;number&gt; tools/apps' phrase found only 12 and 2 in use, both correct: lib/tools/registry.ts TOOLS has exactly 12 entries (extracted the name: fields programmatically -- ids and names both return 12) and PLAN_FEATURES.free.aiToolsAccess = 2. Live: fetched /, /ai-marketing-tools and /contact (all HTTP 200) and regex-extracted every count phrase. Complete set across all three = {12 AI-Powered Marketing Tools, 12 Tools, 12 AI tools, 12 tools, 2 AI tools, 2 tools}. Zero occurrences of 24 or any other count; the has24 regex returned false on all three pages. NEW THIS RUN, and the reason this test needed care rather than a rote grep: the working tree contains an UNCOMMITTED, UNTRACKED 13th user-facing tool -- a GEO/AI-visibility checker (app/geo/, app/api/geo/, lib/geo/, app/dashboard/tools/geo-visibility-checker/). It was deliberately built so as NOT to break the '12 tools' claim: it is not registered in lib/tools/registry.ts, and the redirect stub carries an explicit comment ('this is NOT a 13th entry in lib/tools/registry.ts. TOOLS stays at exactly 12 so every "12 tools" claim in public copy, metadata, JSON-LD and the welcome email remains true'). Verified live that it has not shipped: /geo and /api/geo/scan both return 404 on production. So the count is correct today, but this is now the highest-risk pending change for this test -- the moment /geo ships, the site offers 13 tools to the public while every surface says 12. Flagging for a copy decision BEFORE deploy, not after.</t>
+        </is>
+      </c>
+      <c r="E128" s="31" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="31" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B129" s="31" t="inlineStr">
+        <is>
+          <t>AUTO-002</t>
+        </is>
+      </c>
+      <c r="C129" s="31" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D129" s="22" t="inlineStr">
+        <is>
+          <t>Repo: grep -rn '\$99' across app/, components/, lib/ returned zero matches. Every '$29' and '$199' reconciles to lib/stripe/products.ts (PLAN_FEATURES.pro.price=29 displayed 'Standard'; PLAN_FEATURES.growth.price=199 displayed 'Pro'). Four bare-99 occurrences, all previously documented and all still benign: lib/stripe/products.ts:94-95 enterprise price 99 / annualPrice 950 explicitly commented 'kept for reference, not currently sold' behind comingSoon:true; components/landing/TrustBadges.tsx:7 '99.9% Uptime' in an orphaned unrendered file (see AUTO-016); app/globals.css:19 a CSS lightness value; and the two guard comments at app/page.tsx:22 and app/ai-marketing-tools/page.tsx:42 that record the retired-'99' JSON-LD incident -- both lines themselves read 199, so the 2026-08-23 highPrice fix is still holding. Live: extracted every '$&lt;digits&gt;' token from the three public pages. Homepage = {$0, $29, $278, $199}; /ai-marketing-tools = {$0, $29, $199}; /contact = {$29, $199}. No $99 anywhere. Note on $278: local commit d7b767f ('hide annual') is NOT yet pushed (see AUTO-010 note on unpushed HEAD), so production still renders the $278/yr Standard annual option. That is consistent with what is deployed, not a defect -- but it does mean the annual price, and therefore the stale Stripe price nickname flagged under AUTO-004, is still customer-reachable on the live site.</t>
+        </is>
+      </c>
+      <c r="E129" s="31" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="32" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B130" s="32" t="inlineStr">
+        <is>
+          <t>AUTO-003</t>
+        </is>
+      </c>
+      <c r="C130" s="32" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="D130" s="24" t="inlineStr">
+        <is>
+          <t>CRITICAL. All three defects logged on 2026-08-29 are UNCHANGED -- nothing fixed in the 3 unpushed commits, and no new leak found. (1) app/api/stripe/create-checkout/route.ts:81 still returns `You are already on the ${plan} plan` interpolating the RAW internal key; app/dashboard/billing/page.tsx:216 still renders {error} verbatim into the visible red banner. A $199 customer re-clicking upgrade is shown 'You are already on the growth plan'. Fix is one line: PLAN_DISPLAY_NAME[plan]. First logged 2026-08-22 -- now 5 consecutive runs and 8 days old. (2) lib/email.ts:172 badges every non-free tool with the literal string 'Pro', but all 12 tools unlock on the $29 tier displayed as 'Standard'; the same email's CTA reads 'Unlock all 12 tools for just $29/month'. Reaches every new signup. Correct badge text is 'Standard'. (3) components/dashboard/TopBar.tsx:11 rotating tip still reads 'Pro gives you 200/month across all 12 tools' -- 200/mo is Standard; Pro is 1,500 (PLAN_FEATURES.growth.aiToolsMonthly=1500). Wrong plan name AND understates Pro by 7.5x. Clean elsewhere: the only ${plan}/{userPlan}/{planTier} interpolations in app/ or components/ are (1) plus a harmless success_url query param; PLAN_DISPLAY_NAME is correctly imported and used in admin/users, dashboard/billing, dashboard/page, dashboard/settings, Sidebar and UsageMeter, and lib/stripe/plan-names.ts (the client-safe split made 2026-08-24) is intact. Live plan names on all three public pages are exactly {Free, Standard, Pro, Enterprise}, zero lowercase 'growth' leaks. INVESTIGATED AND CLEARED this run: the automated sweep flagged the capitalized token 'Growth' on the live homepage. Traced it to the single occurrence in the pricing section heading 'Choose Your Growth Plan' (components/landing/Pricing.tsx) -- ordinary marketing copy, not a tier-key leak, so NOT counted as a defect. Worth a note only because that headline sits directly above a card whose displayed name is 'Pro' but whose internal key is 'growth'; the adjacency is unfortunate and a reader could plausibly read 'Growth Plan' as a tier name. Dashboard billing HTML still not diffable unauthenticated (it correctly redirects), so (1),(2),(3) remain code-level verification only.</t>
+        </is>
+      </c>
+      <c r="E130" s="32" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="33" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B131" s="33" t="inlineStr">
+        <is>
+          <t>AUTO-004</t>
+        </is>
+      </c>
+      <c r="C131" s="33" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="D131" s="34" t="inlineStr">
+        <is>
+          <t>BLOCKED -- and this is a Critical-priority test, now blocked on 5 of the last 6 runs. No Stripe MCP connector exists in this session: ToolSearch for stripe/products/prices/billing returns no deferred tools, and mcp__mcp-registry__list_connectors filtered on stripe/payments/billing returns []. Fallbacks also unavailable: the sandbox egress proxy rejects BOTH api.stripe.com and dashboard.stripe.com at CONNECT (HTTP 403, X-Proxy-Error: blocked-by-allowlist); the built-in browser pane refuses to navigate to dashboard.stripe.com ('navigation denied or failed'); and mcp__claude-in-chrome__list_connected_browsers returns [], so there is no authenticated Chrome session to read the dashboard through. DELIBERATELY NOT ATTEMPTED: STRIPE_SECRET_KEY is present in the local .env and could technically have been used from the browser pane's JS context, but injecting a LIVE secret key into a page context is a credential-exposure risk and a security-sensitive action, so it was not done unattended -- flagging the decision rather than silently taking it. Nothing was verified against Stripe this run. Unchanged in the repo, still needing verification: prod_UAltLAeJGLVSqI (price_1TCQLpHTpiuftGGEZWt9UJ2Y, $29, must read 'SHIJO.AI Standard'), prod_UuvJvC2ZKysgfK (price_1Tv5SpHTpiuftGGEMu4TdOzs, $199, must read 'SHIJO.AI Pro'), prod_UAluQCvL32SQ3k (Enterprise, paused). CARRIED FORWARD, still open and unverified: the $278/yr Standard price is nicknamed 'Shijo Pro Annual' and the Enterprise annual price 'Shijo Enterprise Annual' -- retired branding on a price that IS still purchasable (VALID_PLANS.pro.annual) and, per AUTO-002, still rendered on the live homepage. To unblock permanently, connect a Stripe MCP connector; that is the only way this Critical test runs on a genuinely unattended schedule.</t>
+        </is>
+      </c>
+      <c r="E131" s="33" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="31" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B132" s="31" t="inlineStr">
+        <is>
+          <t>AUTO-005</t>
+        </is>
+      </c>
+      <c r="C132" s="31" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D132" s="22" t="inlineStr">
+        <is>
+          <t>Live POST to https://www.shijo.ai/api/auth/register with email 'not-a-valid-email' (name 'Regression Bot', matching valid 12-char passwords so email format was the ONLY invalid field) -&gt; HTTP 400, body {"error":"Please enter a valid email address"}. Not 200; no account created. Method: sandbox curl is still blocked by the egress proxy allowlist (403 X-Proxy-Error: blocked-by-allowlist on CONNECT to www.shijo.ai), but UNLIKE the second 2026-08-29 run the built-in browser pane reached www.shijo.ai successfully this time, so the request was issued as a same-origin fetch with credentials:'omit' from a live page context -- the identical live endpoint, and the same method that produced the passing results on 2026-08-23 and the first 2026-08-29 run.</t>
+        </is>
+      </c>
+      <c r="E132" s="31" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="31" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B133" s="31" t="inlineStr">
+        <is>
+          <t>AUTO-006</t>
+        </is>
+      </c>
+      <c r="C133" s="31" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D133" s="22" t="inlineStr">
+        <is>
+          <t>Live POST to /api/auth/register with password 'ValidPass123!' and confirmPassword 'DifferentPass456!' (throwaway address shijo-regress-20260830a@mailinator.com) -&gt; HTTP 400, body {"error":"Passwords do not match"}. The server-side confirmPassword check shipped 2026-07-19 is still live and still fires ahead of any account creation. No account created. Same same-origin-fetch method as AUTO-005 (sandbox curl blocked by proxy allowlist).</t>
+        </is>
+      </c>
+      <c r="E133" s="31" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="31" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B134" s="31" t="inlineStr">
+        <is>
+          <t>AUTO-007</t>
+        </is>
+      </c>
+      <c r="C134" s="31" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D134" s="22" t="inlineStr">
+        <is>
+          <t>Live POST to /api/auth/register with a 3-character password 'abc' in both password and confirmPassword (throwaway address shijo-regress-20260830b@mailinator.com) -&gt; HTTP 400, body {"error":"Password must be at least 8 characters"}. The 8-character minimum is enforced server-side, independent of the client form. No account created. Same same-origin-fetch method as AUTO-005.</t>
+        </is>
+      </c>
+      <c r="E134" s="31" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="31" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B135" s="31" t="inlineStr">
+        <is>
+          <t>AUTO-008</t>
+        </is>
+      </c>
+      <c r="C135" s="31" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D135" s="22" t="inlineStr">
+        <is>
+          <t>Fetched all 16 protected routes live with credentials:'omit' and redirect:'follow', asserting the final URL landed on /login?redirect=. 16/16 passed -- every one resolved to https://www.shijo.ai/login?redirect=&lt;url-encoded original path&gt;, i.e. a real redirect with the return path preserved, never a 200 carrying authenticated UI. Route list was re-derived this run via `find app/dashboard app/admin -name page.tsx` rather than reused from the last log, which matters because the inventory CHANGED: the new untracked /dashboard/tools/geo-visibility-checker page adds a 16th route (15 last run). It was tested and correctly redirects -- note that even though it is only a redirect stub to the public /geo, middleware.ts intercepts it first, so an anonymous visitor is sent to /login rather than through to /geo. Routes covered -- dashboard: /dashboard, /ai-visibility, /analytics, /billing, /content, /keywords, /settings, /tools, /tools/keyword-research (dynamic [toolId]), /tools/geo-visibility-checker; admin: /admin, /admin/signups, /admin/terms, /admin/tickets, /admin/usage, /admin/users. Matches middleware.ts, matcher ['/dashboard/:path*','/admin/:path*']. (As logged before, app/admin/page.tsx does not exist as a file but the bare /admin path is still covered by the matcher and was verified.)</t>
+        </is>
+      </c>
+      <c r="E135" s="31" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="31" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B136" s="31" t="inlineStr">
+        <is>
+          <t>AUTO-009</t>
+        </is>
+      </c>
+      <c r="C136" s="31" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D136" s="22" t="inlineStr">
+        <is>
+          <t>Fetched all four endpoints live with credentials:'omit', probing BOTH GET and POST on each so nothing leaks on the unintended verb. On their real method all four return 401: /api/usage GET -&gt; 401 {"error":"Not authenticated"}; /api/stripe/create-checkout POST -&gt; 401 {"error":"Please sign in first"}; /api/dashboard/ai-visibility-waitlist POST -&gt; 401 {"success":false,"error":"Please sign in to join the waitlist."}; /api/generate POST -&gt; 401 {"success":false,"error":"Please sign in to use AI tools"}. On the wrong verb each returns 405 with an empty body. No endpoint returned data and no error body disclosed anything beyond the sign-in prompt. ADDED THIS RUN: also probed the new /api/geo/scan route from the untracked GEO feature -- returns 404 on both verbs, confirming it is not deployed. When it does ship it will be a PUBLIC unauthenticated endpoint by design (it is outside the middleware matcher), so it should be added to this test as an explicit exception with its own abuse/rate-limit check rather than a 401 assertion -- lib/geo/budget.ts exists, suggesting spend control was considered, but it was not exercised here.</t>
+        </is>
+      </c>
+      <c r="E136" s="31" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="31" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B137" s="31" t="inlineStr">
+        <is>
+          <t>AUTO-010</t>
+        </is>
+      </c>
+      <c r="C137" s="31" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D137" s="22" t="inlineStr">
+        <is>
+          <t>Read app/api/stripe/create-checkout/route.ts in full. VALID_PLANS keys are exactly {pro, growth}; 'enterprise' is absent with an inline comment recording the 2026-07-19 pause. Cross-checked against lib/stripe/products.ts rather than hardcoding the expected set: PLAN_FEATURES.enterprise carries comingSoon:true and PLAN_FEATURES.free has no priceId, so {pro, growth} is precisely the currently-purchasable set. All three guards present and correct: interval must be monthly|annual (else 400 'Invalid billing interval'); !plan || !VALID_PLANS[plan] -&gt; 400 'Invalid plan selected', catching 'enterprise' and every unrecognized name; and the interval-resolution guard !VALID_PLANS[plan][interval] -&gt; 400 'This plan is not available on that billing interval yet', correctly handling growth having monthly but no annual price. Re-verified the sibling app/api/billing/checkout/route.ts too, since it can also reach Stripe: its ALLOWED_PRICE_IDS is a hand-written list of exactly PRO_MONTHLY, PRO_ANNUAL, GROWTH_MONTHLY -- deliberately not Object.values(STRIPE_PRICE_IDS) -- so the paused ENTERPRISE_* ids are not purchasable there either. IMPORTANT CONTEXT for this whole run: local HEAD is b88b5c0 but origin/main is 48c7a84 -- THREE COMMITS ARE UNPUSHED (b88b5c0 KB update, d7b767f 'D-37 billing-month quota, hide annual, CSP report-only, D-13 atomic upsert', 0f72c97 verification pass), plus 2 modified files and 4 untracked directories. Every repo-side result in this run therefore describes local code, which is AHEAD of production. Note specifically that d7b767f hides the annual option in the UI but does NOT remove pro.annual from VALID_PLANS, so the annual price stays purchasable server-side after that ships -- intentional as far as the code reads, but worth confirming it is what was meant.</t>
+        </is>
+      </c>
+      <c r="E137" s="31" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="31" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B138" s="31" t="inlineStr">
+        <is>
+          <t>AUTO-011</t>
+        </is>
+      </c>
+      <c r="C138" s="31" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D138" s="22" t="inlineStr">
+        <is>
+          <t>Fetched https://www.shijo.ai/sitemap.xml live -- HTTP 200, 13 &lt;loc&gt; entries, zero matches for 'dashboard' or 'admin'. Full list: /blog plus 3 blog posts (ai-seo-tools-keyword-research-faster, ai-ad-copy-that-converts, ai-marketing-tools-small-business-2026), the root, /contact, /ai-marketing-tools, and the 6 legal pages (/terms, /privacy, /cookies, /gdpr-compliance, /ai-compliance, /security). Identical to 2026-08-29. Consistent with AUTO-008: the routes middleware.ts bounces to /login are also absent from the crawlable sitemap, so there is no information-disclosure path via search. PENDING CHANGE, verified safe: app/sitemap.ts is modified locally to add ONE new public URL, https://www.shijo.ai/geo, priority 0.8. That is a genuinely public unauthenticated route, so it is not a leak -- and the diff comment explicitly records that /pricing and /features were deliberately NOT added because they 404 on production, which I confirmed live (both return 404). Re-check this test after the geo deploy: /geo itself currently 404s live, so the entry must not ship ahead of the page or the sitemap will advertise a dead URL to crawlers.</t>
+        </is>
+      </c>
+      <c r="E138" s="31" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="32" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B139" s="32" t="inlineStr">
+        <is>
+          <t>AUTO-013</t>
+        </is>
+      </c>
+      <c r="C139" s="32" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="D139" s="24" t="inlineStr">
+        <is>
+          <t>Both previously-logged violations persist, and there is a THIRD, new, unshipped one. (1) STILL LIVE in public marketing copy, now 42 days old (since commit fcd06fa, 2026-07-19): components/landing/Pricing.tsx renders '2 AI tools (Haiku-powered)' (line 27) and 'Sonnet AI for complex tasks' (lines 48 and 69). Re-confirmed live this run -- a regex sweep for /claude|anthropic|haiku|sonnet|opus/i over the rendered HTML of all three public pages returns {Haiku, Sonnet} on the homepage and NOTHING on /ai-marketing-tools or /contact. Haiku and Sonnet are Claude model names, so the homepage names the AI vendor in customer-facing copy, which the product rule confines to /privacy, /security and /ai-compliance. The compliant wording already exists in the repo -- components/lp/LandingPageContent.tsx says 'Advanced AI for complex tasks', which is exactly what /ai-marketing-tools serves live -- so the fix is to copy that phrasing into Pricing.tsx lines 27/48/69. Repeating the recommendation from the last two runs: the sheet's own Method grep ('claude|anthropic') CANNOT catch this and should be widened to 'claude|anthropic|haiku|sonnet|opus'. (2) PERSISTS, unchanged since 2026-07-20: app/gdpr-compliance/page.tsx:77 renders public text 'Anthropic -- AI model infrastructure powering platform features'. Still a policy-scope decision for Sri, not a code bug: either formally add /gdpr-compliance as a fourth approved disclosure location (defensible -- it is a legal page listing sub-processors, exactly the carve-out the rule intends) or drop the vendor name. (3) NEW, NOT YET LIVE, needs an explicit decision before the GEO feature deploys: the untracked GEO checker names Claude in customer-facing product UI. lib/geo/types.ts:42 sets ENGINE_LABELS.claude = 'Claude', which GeoChecker.tsx renders as a column header in the results grid, and app/geo/page.tsx's meta description reads '...whether ChatGPT, Gemini, Perplexity, Claude and Google AI Overviews mention your business...'. The developer anticipated this and left a rationale comment above ENGINE_LABELS arguing these labels name engines the USER asked us to query, which is a different thing from disclosing the vendor behind the 12 tools. That reasoning is sound and I am not overriding it -- but it is a new interpretation of a rule Sri wrote, so it needs Sri's explicit sign-off rather than a code comment's, especially since app/layout.tsx:14-16 documents a PRIOR incident with near-identical wording ('track your visibility in ChatGPT, Claude &amp; Perplexity') that was treated as a violation and removed on 2026-07-18. Also note lib/geo/engines/claude.ts reuses the same ANTHROPIC_API_KEY that powers the 12 dashboard tools, so the vendor genuinely is both a measured engine and the underlying supplier. Confirmed non-violations (backend or non-rendered, unchanged): app/api/generate/route.ts SDK import + model-id constants + one comment, lib/ai/claude.ts (entirely backend plumbing), lib/ai/pricing.ts model-id cost keys, lib/tools/usage.ts:50 comment, app/layout.tsx:14-16 comment, app/robots.ts:20 'Claude-Web' crawler directive, and the internal haiku/sonnet modelTier enums that ToolPage.tsx and dashboard/tools map to the neutral labels Fast/Advanced.</t>
+        </is>
+      </c>
+      <c r="E139" s="32" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="31" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B140" s="31" t="inlineStr">
+        <is>
+          <t>AUTO-015</t>
+        </is>
+      </c>
+      <c r="C140" s="31" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D140" s="22" t="inlineStr">
+        <is>
+          <t>Diffed programmatically: regex-extracted the tool names from buildWelcomeEmail() in lib/email.ts and from the TOOLS export in lib/tools/registry.ts, compared as sets in both directions. 12 names each side, symmetric difference empty. Exact match: Post Caption Generator, Keyword Research, SEO Content Brief, SEO Meta Generator, FAQ Generator, AI Overview Optimizer, Ad Copy Generator, Ad Headline A/B Tester, Audience Targeting Profiles, Landing Page Copy Generator, Email Sequence Generator, Newsletter Generator. (Order differs because the email groups by category -- expected, not a mismatch.) The free/paid split is also correct and was checked separately: the two tools badged FREE in the email (Post Caption Generator, SEO Meta Generator) are exactly the two registry entries with minPlan:'free'. The 24-fabricated-name regression fixed 2026-07-19 has not returned, and the hand-sync warning comment at lib/email.ts:135-139 is still in place. TWO CARRY-FORWARD NOTES: (a) the paid-tool badge TEXT in this same email is wrong ('Pro' where it should read 'Standard') -- logged under AUTO-003, not a tool-list mismatch, so it does not change this result; (b) this test is hand-synced by design, and the pending GEO checker is the next thing likely to break it -- if /geo ships and is ever mentioned in the welcome email without being added to registry.ts, this diff fails. It correctly is NOT in the email today.</t>
+        </is>
+      </c>
+      <c r="E140" s="31" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="32" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B141" s="32" t="inlineStr">
+        <is>
+          <t>AUTO-016</t>
+        </is>
+      </c>
+      <c r="C141" s="32" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="D141" s="24" t="inlineStr">
+        <is>
+          <t>One item live, two latent, one dormant, plus one NEW latent claim. (1) STILL FAILING, 5th consecutive run since 2026-08-22: components/landing/UseCases.tsx:24 renders 'Trusted by marketing teams, agencies, and brands worldwide' under a 'Built for Modern Enterprises' heading -- re-confirmed verbatim in the live homepage HTML this run, and it is the ONLY claim the live sweep surfaced across all three public pages. Unverifiable social proof (plural teams, agencies, brands, worldwide). The customer count could not be re-checked this run (AUTO-004 blocked, no DB access); the last actual reading, 2026-08-29, was 1 active subscription on Standard, which does not substantiate the wording. Needs Sri to soften the copy or confirm real customers -- not safely auto-fixable. (2) LATENT, unchanged: lib/seo-config.ts pages.features (lines 38-41) and pages.dashboard (lines 50-52) describe unbuilt capabilities as shipped -- 'clustering, intent classification, search volume checking, SERP analysis, and rank tracking', 'Enterprise-grade SEO tools', 'measuring AI search visibility', 'Real-time SEO analytics'. Both also declare canonicals pointing at /features and /dashboard; I verified live that /features returns 404, so those canonicals are dead. pages.pricing additionally still says 'Free, Pro &amp; Enterprise Plans' though Enterprise is paused, and its canonical /pricing is also a live 404. Nothing renders from these today (only pages.home is wired up) but any future generatePageMetadata('features'|'dashboard'|'pricing') call publishes fabricated claims and dead canonicals instantly. Recommend deleting the dead entries rather than leaving the trap -- note app/geo/page.tsx's own comment says the author avoided this file precisely because it is 'under an ads freeze' and its canonicals point at 404s, so the trap is now actively shaping how new code gets written. (3) STILL DORMANT: components/landing/TrustBadges.tsx retains 'SOC 2 Compliant', '99.9% Uptime', '10M+ Keywords Analyzed Daily', '500+ Enterprises'. grep across app/, components/, lib/ finds the identifier only in its own definition file -- zero imports -- and none of the four strings appear in the live HTML of any public page. Still needs a user-run rm; the sandbox cannot delete. (4) NEW, LATENT, in the untracked GEO checker: app/geo/page.tsx tells visitors 'We ask five answer engines the questions your customers actually ask' and GeoChecker.tsx's button reads 'Checking five engines...' -- both hardcode FIVE. But of the five adapters only claude.ts has its key present (ANTHROPIC_API_KEY); the local .env/.env.local contain no OPENAI_API_KEY, GEMINI_API_KEY, PERPLEXITY_API_KEY, DATAFORSEO_LOGIN/PASSWORD or GOOGLE_PLACES_API_KEY. Production env vars live in Vercel and could not be read from here, so this is NOT confirmed as a production defect -- but if those keys are absent at deploy, the page promises five engines and delivers one. Mitigating: lib/geo/orchestrator.ts degrades properly, recording unavailable engines as 'skipped' with 'Not checked -- engine unavailable' rather than scoring them as negatives, and the UI surfaces a degraded-engines notice. Recommended before shipping: confirm all five keys exist in production, or make the count dynamic from the available-adapter list instead of hardcoding 'five'. (5) CLEAN: app/layout.tsx metadata describes the real 12-tool product and claims no certifications; app/page.tsx JSON-LD omits aggregateRating and reports offerCount 3 / highPrice 199.</t>
+        </is>
+      </c>
+      <c r="E141" s="32" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix build: drop duplicate Window.dataLayer declaration in PurchaseTracker
components/CookieConsentBanner.tsx already declares Window.dataLayer globally
as unknown[]. PurchaseTracker redeclared it as Record<string, unknown>[], and
TypeScript merges global interfaces across the whole project, so the two
conflicted: TS2717 'Subsequent property declarations must have the same type'.
Vercel failed the build on 9960085.

Removed the redeclaration and used the existing global. Pushing an object into
unknown[] is fine, so nothing else changed.

Root cause on my side: I verified the file in isolation with tsc --noResolve,
which by construction cannot see cross-file 'declare global' merging. Verified
this fix by typechecking PurchaseTracker and CookieConsentBanner TOGETHER, and
confirmed that check is real by re-introducing the bad declaration and watching
it reproduce the same TS2717.
</commit_message>
<xml_diff>
--- a/docs/testing/Automated-Regression-Test-Suite.xlsx
+++ b/docs/testing/Automated-Regression-Test-Suite.xlsx
@@ -152,7 +152,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -242,6 +242,21 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1476,7 +1491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E141"/>
+  <dimension ref="A1:E169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3377,17 +3392,17 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="21" t="inlineStr">
+      <c r="A71" s="35" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B71" s="21" t="inlineStr">
+      <c r="B71" s="35" t="inlineStr">
         <is>
           <t>AUTO-001</t>
         </is>
       </c>
-      <c r="C71" s="21" t="inlineStr">
+      <c r="C71" s="35" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -3397,24 +3412,24 @@
           <t>Repo: grep -rniE '24.{0,15}(tools|apps)' across app/, components/, lib/ returned zero matches; every numeric tool claim in source is '12' (seo-config.ts, layout.tsx, email.ts, LandingPageContent.tsx, Pricing.tsx, Hero.tsx, Features.tsx). lib/tools/registry.ts TOOLS export contains exactly 12 tool objects. Live: homepage shows '12 AI-Powered Marketing Tools' / '12 Tools, One Platform' with 12 tool cards rendered; /ai-marketing-tools shows '12 AI-Powered Marketing Tools' / '12 Tools Across 4 Categories' / 'Choose from 12 tools'; /contact shows '12 Tools, One Platform' and 'Standard: $29/mo, all 12 tools'. No fabricated tool count anywhere.</t>
         </is>
       </c>
-      <c r="E71" s="21" t="inlineStr">
+      <c r="E71" s="35" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="23" t="inlineStr">
+      <c r="A72" s="36" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B72" s="23" t="inlineStr">
+      <c r="B72" s="36" t="inlineStr">
         <is>
           <t>AUTO-002</t>
         </is>
       </c>
-      <c r="C72" s="23" t="inlineStr">
+      <c r="C72" s="36" t="inlineStr">
         <is>
           <t>Fail</t>
         </is>
@@ -3424,24 +3439,24 @@
           <t>CRITICAL, STILL UNFIXED -- now 34 days stale live (code corrected 2026-07-19; first logged as a live failure 2026-08-11, unchanged since). Live https://www.shijo.ai/ai-marketing-tools still serves the pre-restructure pricing table: 'Pro $29/month' and 'Enterprise $99/month' with an active 'Get Started with Enterprise' CTA linking to /register -- a plan that cannot be purchased (VALID_PLANS in create-checkout excludes enterprise), so anyone clicking it hits a dead end. Code is clean and shipped: grep '$99' across app/, components/, lib/ = zero matches; git HEAD == origin/main == 765afda; git show origin/main:components/lp/LandingPageContent.tsx confirms the committed file has Standard $29 / Pro $199 / Enterprise 'Coming Soon'; the file has no uncommitted local diff. So this is a deployment/CDN-cache gap on the /ai-marketing-tools route, not a code bug -- root cause not diagnosable from this sandbox (no Vercel/hosting access). Needs a redeploy or cache purge of that route. Homepage and /contact both correct ($29 Standard, $199 Pro, Enterprise 'Coming Soon', no $99). Separately re-confirmed: app/page.tsx:22 and app/ai-marketing-tools/page.tsx:37 both still hardcode JSON-LD offers.highPrice:'99' (should be '199').</t>
         </is>
       </c>
-      <c r="E72" s="23" t="inlineStr">
+      <c r="E72" s="36" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="23" t="inlineStr">
+      <c r="A73" s="36" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B73" s="23" t="inlineStr">
+      <c r="B73" s="36" t="inlineStr">
         <is>
           <t>AUTO-003</t>
         </is>
       </c>
-      <c r="C73" s="23" t="inlineStr">
+      <c r="C73" s="36" t="inlineStr">
         <is>
           <t>Fail</t>
         </is>
@@ -3451,24 +3466,24 @@
           <t>CRITICAL. (a) Live: the same stale /ai-marketing-tools page names the $29 tier 'Pro' instead of 'Standard' (PLAN_DISPLAY_NAME.pro='Standard'), directly contradicting the homepage and /contact, which both correctly say 'Standard' for $29 and 'Pro' for $199. Same stale-deployment root cause as AUTO-002. (b) NEW code-level finding not previously logged: app/api/stripe/create-checkout/route.ts:81 returns `You are already on the ${plan} plan` interpolating the RAW internal key, and app/dashboard/billing/page.tsx:108 renders data.error verbatim into the visible red error banner (line 181) -- so a customer on the $199 tier who re-clicks upgrade sees 'You are already on the growth plan'. Should be PLAN_DISPLAY_NAME[plan]. All 6 other user-facing plan-name surfaces are correct (admin/users, dashboard/billing x3, dashboard/page, dashboard/settings, UsageMeter all import PLAN_DISPLAY_NAME). Dashboard billing page HTML could not be diffed live -- it correctly redirects to /login when unauthenticated -- so (b) is verified at code level only. Also noted (not a failure, dead branch): components/dashboard/ToolPage.tsx:192 and lib/tools/usage.ts:116 fall back to the string 'Enterprise' as the upgrade target, but all 12 registry tools have minPlan of 'free' or 'pro', so that branch is unreachable today; it would surface a paused plan as purchasable if a tool were ever gated above 'pro'.</t>
         </is>
       </c>
-      <c r="E73" s="23" t="inlineStr">
+      <c r="E73" s="36" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="25" t="inlineStr">
+      <c r="A74" s="37" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B74" s="25" t="inlineStr">
+      <c r="B74" s="37" t="inlineStr">
         <is>
           <t>AUTO-004</t>
         </is>
       </c>
-      <c r="C74" s="25" t="inlineStr">
+      <c r="C74" s="37" t="inlineStr">
         <is>
           <t>Blocked</t>
         </is>
@@ -3478,24 +3493,24 @@
           <t>Could not run. No Stripe MCP tools are available in this session -- ToolSearch for 'stripe products prices' returned 'No matching deferred tools found'. Second consecutive scheduled run blocked on this (also blocked 2026-08-11); the 07-20 through 07-22 runs had Stripe access and passed. Stripe Product .name drift against PLAN_DISPLAY_NAME (prod_UAltLAeJGLVSqI must read 'SHIJO.AI Standard', prod_UuvJvC2ZKysgfK 'SHIJO.AI Pro') is therefore unverified for 11 days. This is the check that caught the live 'Shijo Pro' mislabel on 2026-07-19, and it is invisible to any code review -- worth reconnecting the Stripe connector.</t>
         </is>
       </c>
-      <c r="E74" s="25" t="inlineStr">
+      <c r="E74" s="37" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="21" t="inlineStr">
+      <c r="A75" s="35" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B75" s="21" t="inlineStr">
+      <c r="B75" s="35" t="inlineStr">
         <is>
           <t>AUTO-005</t>
         </is>
       </c>
-      <c r="C75" s="21" t="inlineStr">
+      <c r="C75" s="35" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -3505,24 +3520,24 @@
           <t>Ran live against https://www.shijo.ai/api/auth/register via a same-origin fetch with credentials:'omit' (the sandbox proxy still blocks direct curl to shijo.ai with 403 blocked-by-allowlist, so this was executed through the connected Chrome session instead -- first time this test has actually run live since 2026-07-22). POST {email:'not-an-email', password:'ValidPass123!', confirmPassword:same} returned HTTP 400 with {"error":"Please enter a valid email address"}. No account created.</t>
         </is>
       </c>
-      <c r="E75" s="21" t="inlineStr">
+      <c r="E75" s="35" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="21" t="inlineStr">
+      <c r="A76" s="35" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B76" s="21" t="inlineStr">
+      <c r="B76" s="35" t="inlineStr">
         <is>
           <t>AUTO-006</t>
         </is>
       </c>
-      <c r="C76" s="21" t="inlineStr">
+      <c r="C76" s="35" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -3532,24 +3547,24 @@
           <t>Live POST to /api/auth/register (same method as AUTO-005) with email shijo-regtest-mismatch-20260822@mailinator.com, password 'ValidPass123!' vs confirmPassword 'DifferentPass456!' returned HTTP 400 with {"error":"Passwords do not match"}. Server-side mismatch check shipped 2026-07-19 is still live. No account created.</t>
         </is>
       </c>
-      <c r="E76" s="21" t="inlineStr">
+      <c r="E76" s="35" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="21" t="inlineStr">
+      <c r="A77" s="35" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B77" s="21" t="inlineStr">
+      <c r="B77" s="35" t="inlineStr">
         <is>
           <t>AUTO-007</t>
         </is>
       </c>
-      <c r="C77" s="21" t="inlineStr">
+      <c r="C77" s="35" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -3559,24 +3574,24 @@
           <t>Live POST to /api/auth/register with a 3-character password ('abc'/'abc', email shijo-regtest-weak-20260822@mailinator.com) returned HTTP 400 with {"error":"Password must be at least 8 characters"}. 8-char minimum enforced server-side. No account created.</t>
         </is>
       </c>
-      <c r="E77" s="21" t="inlineStr">
+      <c r="E77" s="35" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="21" t="inlineStr">
+      <c r="A78" s="35" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B78" s="21" t="inlineStr">
+      <c r="B78" s="35" t="inlineStr">
         <is>
           <t>AUTO-008</t>
         </is>
       </c>
-      <c r="C78" s="21" t="inlineStr">
+      <c r="C78" s="35" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -3586,24 +3601,24 @@
           <t>Fetched all 13 protected routes live with credentials:'omit' (no session cookie): /admin, /admin/terms, /admin/tickets, /admin/users, /dashboard, /dashboard/ai-visibility, /dashboard/analytics, /dashboard/billing, /dashboard/content, /dashboard/keywords, /dashboard/settings, /dashboard/tools, /dashboard/tools/keyword-research. Every one redirected (redirect:'manual' gave type 'opaqueredirect' for all 13; follow mode resolved each to /login?redirect=&lt;url-encoded original path&gt;) and every response body was the identical 12,779-byte login page -- zero authenticated UI leaked. Matches middleware.ts matcher ['/dashboard/:path*','/admin/:path*']. Full route-by-route live verification achieved this run (prior run was Blocked/partial).</t>
         </is>
       </c>
-      <c r="E78" s="21" t="inlineStr">
+      <c r="E78" s="35" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="21" t="inlineStr">
+      <c r="A79" s="35" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B79" s="21" t="inlineStr">
+      <c r="B79" s="35" t="inlineStr">
         <is>
           <t>AUTO-009</t>
         </is>
       </c>
-      <c r="C79" s="21" t="inlineStr">
+      <c r="C79" s="35" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -3613,24 +3628,24 @@
           <t>Fetched all 4 endpoints live with credentials:'omit', using the correct HTTP verb for each (POST for the three POST-only routes, which a GET-only fetcher could not previously reach): /api/usage GET -&gt; 401 {"error":"Not authenticated"}; /api/stripe/create-checkout POST -&gt; 401 {"error":"Please sign in first"}; /api/dashboard/ai-visibility-waitlist POST -&gt; 401 {"success":false,"error":"Please sign in to join the waitlist."}; /api/generate POST -&gt; 401 {"success":false,"error":"Please sign in to use AI tools"}. All four correctly reject anonymous requests. First fully-live run of this test (Blocked 2026-08-11).</t>
         </is>
       </c>
-      <c r="E79" s="21" t="inlineStr">
+      <c r="E79" s="35" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="21" t="inlineStr">
+      <c r="A80" s="35" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B80" s="21" t="inlineStr">
+      <c r="B80" s="35" t="inlineStr">
         <is>
           <t>AUTO-010</t>
         </is>
       </c>
-      <c r="C80" s="21" t="inlineStr">
+      <c r="C80" s="35" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -3640,24 +3655,24 @@
           <t>Read app/api/stripe/create-checkout/route.ts: VALID_PLANS keys are exactly {pro, growth}. Reconciled against lib/stripe/products.ts -- PLAN_FEATURES.enterprise carries comingSoon:true (paused), free is not a paid tier, so {pro, growth} is precisely the currently-purchasable set. 'enterprise' and any unrecognized plan name fall through to the 400 'Invalid plan selected' branch (lines 49-54). Interval guard present at lines 56-62: growth has no annual priceId, so plan:'growth'+interval:'annual' correctly 400s rather than passing undefined to Stripe. Auth 401 check runs before any plan validation. Verified live in AUTO-009 that the endpoint 401s anonymously.</t>
         </is>
       </c>
-      <c r="E80" s="21" t="inlineStr">
+      <c r="E80" s="35" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="21" t="inlineStr">
+      <c r="A81" s="35" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B81" s="21" t="inlineStr">
+      <c r="B81" s="35" t="inlineStr">
         <is>
           <t>AUTO-011</t>
         </is>
       </c>
-      <c r="C81" s="21" t="inlineStr">
+      <c r="C81" s="35" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -3667,24 +3682,24 @@
           <t>Fetched https://www.shijo.ai/sitemap.xml live -- readable XML this run (previous runs returned an unreadable binary body). 13 &lt;loc&gt; entries: /blog, 3 blog posts, homepage, /terms, /privacy, /cookies, /gdpr-compliance, /ai-compliance, /security, /contact, /ai-marketing-tools. Zero /dashboard and zero /admin URLs. Live contents independently confirmed against app/sitemap.ts for the first time.</t>
         </is>
       </c>
-      <c r="E81" s="21" t="inlineStr">
+      <c r="E81" s="35" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="23" t="inlineStr">
+      <c r="A82" s="36" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B82" s="23" t="inlineStr">
+      <c r="B82" s="36" t="inlineStr">
         <is>
           <t>AUTO-013</t>
         </is>
       </c>
-      <c r="C82" s="23" t="inlineStr">
+      <c r="C82" s="36" t="inlineStr">
         <is>
           <t>Fail</t>
         </is>
@@ -3694,24 +3709,24 @@
           <t>PERSISTS, unchanged since 2026-07-20 (now 33 days). grep -rin 'claude|anthropic' across app/, components/, lib/ excluding /privacy, /security, /ai-compliance returns the same set as every prior run. Non-violations (backend code and non-rendered text, unchanged): app/api/generate/route.ts (SDK import, model ID strings, a code comment), lib/ai/claude.ts (entire module is backend SDK plumbing), lib/tools/usage.ts:49 (code comment), app/layout.tsx:14-16 (code comment documenting a past fix), app/robots.ts:20 ('Claude-Web' crawler allow-directive alongside GPTBot/PerplexityBot -- technical SEO). The one real violation, still unresolved: app/gdpr-compliance/page.tsx:76 renders visible public text 'Anthropic -- AI model infrastructure powering platform features' on /gdpr-compliance, which is not one of the three approved disclosure locations. Still awaiting Sri's decision: either add /gdpr-compliance as a fourth approved location (defensible -- it is a legal/compliance page listing sub-processors, exactly the context the rule carves out) or drop the vendor name there. This is a policy-scope question, not a code bug; it will keep failing every run until the rule or the page changes.</t>
         </is>
       </c>
-      <c r="E82" s="23" t="inlineStr">
+      <c r="E82" s="36" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="21" t="inlineStr">
+      <c r="A83" s="35" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B83" s="21" t="inlineStr">
+      <c r="B83" s="35" t="inlineStr">
         <is>
           <t>AUTO-015</t>
         </is>
       </c>
-      <c r="C83" s="21" t="inlineStr">
+      <c r="C83" s="35" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -3721,24 +3736,24 @@
           <t>Diffed lib/email.ts buildWelcomeEmail() against lib/tools/registry.ts TOOLS export. Both list exactly 12 tools, name-for-name with no extras or omissions: Post Caption Generator, SEO Meta Generator, Keyword Research, SEO Content Brief, FAQ Generator, AI Overview Optimizer, Ad Copy Generator, Ad Headline A/B Tester, Audience Targeting Profiles, Landing Page Copy Generator, Email Sequence Generator, Newsletter Generator. Also verified the email's free:true flags (Post Caption Generator, SEO Meta Generator) match the two registry entries with minPlan:'free' -- so the email does not promise free access to a gated tool. No drift since the 2026-07-19 fix.</t>
         </is>
       </c>
-      <c r="E83" s="21" t="inlineStr">
+      <c r="E83" s="35" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="23" t="inlineStr">
+      <c r="A84" s="36" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B84" s="23" t="inlineStr">
+      <c r="B84" s="36" t="inlineStr">
         <is>
           <t>AUTO-016</t>
         </is>
       </c>
-      <c r="C84" s="23" t="inlineStr">
+      <c r="C84" s="36" t="inlineStr">
         <is>
           <t>Fail</t>
         </is>
@@ -3748,7 +3763,7 @@
           <t>Marking Fail this run where 08-11 logged the same core evidence as Pass-with-note; calling it a failure because the item is a false claim shipped in machine-readable metadata on two live public pages, which is exactly this test's remit. (1) app/page.tsx:22 and app/ai-marketing-tools/page.tsx:37 publish JSON-LD AggregateOffer highPrice:'99' -- asserting to Google that a $99 tier is currently purchasable. It is not: Enterprise is paused (comingSoon:true) and excluded from VALID_PLANS. Correct value is '199'. (2) NEW, not previously flagged: components/landing/UseCases.tsx:24 renders 'Trusted by marketing teams, agencies, and brands worldwide' live on the homepage under a 'Built for Modern Enterprises' heading. That is an unverifiable social-proof claim, and lib/stripe/products.ts documents zero customers on any plan as of 2026-07-19; current customer count could not be checked this run (no Stripe MCP, no DB access), so this needs Sri to confirm or soften the wording rather than being auto-fixable. (3) Unchanged and still clean: components/landing/TrustBadges.tsx retains fabricated 'SOC 2 Compliant' / '99.9% Uptime' / '10M+ Keywords' / '500+ Enterprises' badges but remains orphaned -- grep across app/ and components/ finds zero imports, and none of that text appears in the live homepage, /ai-marketing-tools, or /contact HTML fetched this run. app/layout.tsx metadata and lib/seo-config.ts are clean (12-tool product described accurately, no certifications claimed); app/page.tsx JSON-LD still correctly omits aggregateRating.</t>
         </is>
       </c>
-      <c r="E84" s="23" t="inlineStr">
+      <c r="E84" s="36" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -4916,17 +4931,17 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="31" t="inlineStr">
+      <c r="A128" s="35" t="inlineStr">
         <is>
           <t>2026-08-30</t>
         </is>
       </c>
-      <c r="B128" s="31" t="inlineStr">
+      <c r="B128" s="35" t="inlineStr">
         <is>
           <t>AUTO-001</t>
         </is>
       </c>
-      <c r="C128" s="31" t="inlineStr">
+      <c r="C128" s="35" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -4936,24 +4951,24 @@
           <t>Repo: grep -rniE '24[^0-9]{0,15}(tools|apps)' across app/, components/, lib/ returned ZERO matches. Broader sweep for any '&lt;number&gt; tools/apps' phrase found only 12 and 2 in use, both correct: lib/tools/registry.ts TOOLS has exactly 12 entries (extracted the name: fields programmatically -- ids and names both return 12) and PLAN_FEATURES.free.aiToolsAccess = 2. Live: fetched /, /ai-marketing-tools and /contact (all HTTP 200) and regex-extracted every count phrase. Complete set across all three = {12 AI-Powered Marketing Tools, 12 Tools, 12 AI tools, 12 tools, 2 AI tools, 2 tools}. Zero occurrences of 24 or any other count; the has24 regex returned false on all three pages. NEW THIS RUN, and the reason this test needed care rather than a rote grep: the working tree contains an UNCOMMITTED, UNTRACKED 13th user-facing tool -- a GEO/AI-visibility checker (app/geo/, app/api/geo/, lib/geo/, app/dashboard/tools/geo-visibility-checker/). It was deliberately built so as NOT to break the '12 tools' claim: it is not registered in lib/tools/registry.ts, and the redirect stub carries an explicit comment ('this is NOT a 13th entry in lib/tools/registry.ts. TOOLS stays at exactly 12 so every "12 tools" claim in public copy, metadata, JSON-LD and the welcome email remains true'). Verified live that it has not shipped: /geo and /api/geo/scan both return 404 on production. So the count is correct today, but this is now the highest-risk pending change for this test -- the moment /geo ships, the site offers 13 tools to the public while every surface says 12. Flagging for a copy decision BEFORE deploy, not after.</t>
         </is>
       </c>
-      <c r="E128" s="31" t="inlineStr">
+      <c r="E128" s="35" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="31" t="inlineStr">
+      <c r="A129" s="35" t="inlineStr">
         <is>
           <t>2026-08-30</t>
         </is>
       </c>
-      <c r="B129" s="31" t="inlineStr">
+      <c r="B129" s="35" t="inlineStr">
         <is>
           <t>AUTO-002</t>
         </is>
       </c>
-      <c r="C129" s="31" t="inlineStr">
+      <c r="C129" s="35" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -4963,24 +4978,24 @@
           <t>Repo: grep -rn '\$99' across app/, components/, lib/ returned zero matches. Every '$29' and '$199' reconciles to lib/stripe/products.ts (PLAN_FEATURES.pro.price=29 displayed 'Standard'; PLAN_FEATURES.growth.price=199 displayed 'Pro'). Four bare-99 occurrences, all previously documented and all still benign: lib/stripe/products.ts:94-95 enterprise price 99 / annualPrice 950 explicitly commented 'kept for reference, not currently sold' behind comingSoon:true; components/landing/TrustBadges.tsx:7 '99.9% Uptime' in an orphaned unrendered file (see AUTO-016); app/globals.css:19 a CSS lightness value; and the two guard comments at app/page.tsx:22 and app/ai-marketing-tools/page.tsx:42 that record the retired-'99' JSON-LD incident -- both lines themselves read 199, so the 2026-08-23 highPrice fix is still holding. Live: extracted every '$&lt;digits&gt;' token from the three public pages. Homepage = {$0, $29, $278, $199}; /ai-marketing-tools = {$0, $29, $199}; /contact = {$29, $199}. No $99 anywhere. Note on $278: local commit d7b767f ('hide annual') is NOT yet pushed (see AUTO-010 note on unpushed HEAD), so production still renders the $278/yr Standard annual option. That is consistent with what is deployed, not a defect -- but it does mean the annual price, and therefore the stale Stripe price nickname flagged under AUTO-004, is still customer-reachable on the live site.</t>
         </is>
       </c>
-      <c r="E129" s="31" t="inlineStr">
+      <c r="E129" s="35" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="32" t="inlineStr">
+      <c r="A130" s="36" t="inlineStr">
         <is>
           <t>2026-08-30</t>
         </is>
       </c>
-      <c r="B130" s="32" t="inlineStr">
+      <c r="B130" s="36" t="inlineStr">
         <is>
           <t>AUTO-003</t>
         </is>
       </c>
-      <c r="C130" s="32" t="inlineStr">
+      <c r="C130" s="36" t="inlineStr">
         <is>
           <t>Fail</t>
         </is>
@@ -4990,7 +5005,7 @@
           <t>CRITICAL. All three defects logged on 2026-08-29 are UNCHANGED -- nothing fixed in the 3 unpushed commits, and no new leak found. (1) app/api/stripe/create-checkout/route.ts:81 still returns `You are already on the ${plan} plan` interpolating the RAW internal key; app/dashboard/billing/page.tsx:216 still renders {error} verbatim into the visible red banner. A $199 customer re-clicking upgrade is shown 'You are already on the growth plan'. Fix is one line: PLAN_DISPLAY_NAME[plan]. First logged 2026-08-22 -- now 5 consecutive runs and 8 days old. (2) lib/email.ts:172 badges every non-free tool with the literal string 'Pro', but all 12 tools unlock on the $29 tier displayed as 'Standard'; the same email's CTA reads 'Unlock all 12 tools for just $29/month'. Reaches every new signup. Correct badge text is 'Standard'. (3) components/dashboard/TopBar.tsx:11 rotating tip still reads 'Pro gives you 200/month across all 12 tools' -- 200/mo is Standard; Pro is 1,500 (PLAN_FEATURES.growth.aiToolsMonthly=1500). Wrong plan name AND understates Pro by 7.5x. Clean elsewhere: the only ${plan}/{userPlan}/{planTier} interpolations in app/ or components/ are (1) plus a harmless success_url query param; PLAN_DISPLAY_NAME is correctly imported and used in admin/users, dashboard/billing, dashboard/page, dashboard/settings, Sidebar and UsageMeter, and lib/stripe/plan-names.ts (the client-safe split made 2026-08-24) is intact. Live plan names on all three public pages are exactly {Free, Standard, Pro, Enterprise}, zero lowercase 'growth' leaks. INVESTIGATED AND CLEARED this run: the automated sweep flagged the capitalized token 'Growth' on the live homepage. Traced it to the single occurrence in the pricing section heading 'Choose Your Growth Plan' (components/landing/Pricing.tsx) -- ordinary marketing copy, not a tier-key leak, so NOT counted as a defect. Worth a note only because that headline sits directly above a card whose displayed name is 'Pro' but whose internal key is 'growth'; the adjacency is unfortunate and a reader could plausibly read 'Growth Plan' as a tier name. Dashboard billing HTML still not diffable unauthenticated (it correctly redirects), so (1),(2),(3) remain code-level verification only.</t>
         </is>
       </c>
-      <c r="E130" s="32" t="inlineStr">
+      <c r="E130" s="36" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -5024,17 +5039,17 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="31" t="inlineStr">
+      <c r="A132" s="35" t="inlineStr">
         <is>
           <t>2026-08-30</t>
         </is>
       </c>
-      <c r="B132" s="31" t="inlineStr">
+      <c r="B132" s="35" t="inlineStr">
         <is>
           <t>AUTO-005</t>
         </is>
       </c>
-      <c r="C132" s="31" t="inlineStr">
+      <c r="C132" s="35" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -5044,24 +5059,24 @@
           <t>Live POST to https://www.shijo.ai/api/auth/register with email 'not-a-valid-email' (name 'Regression Bot', matching valid 12-char passwords so email format was the ONLY invalid field) -&gt; HTTP 400, body {"error":"Please enter a valid email address"}. Not 200; no account created. Method: sandbox curl is still blocked by the egress proxy allowlist (403 X-Proxy-Error: blocked-by-allowlist on CONNECT to www.shijo.ai), but UNLIKE the second 2026-08-29 run the built-in browser pane reached www.shijo.ai successfully this time, so the request was issued as a same-origin fetch with credentials:'omit' from a live page context -- the identical live endpoint, and the same method that produced the passing results on 2026-08-23 and the first 2026-08-29 run.</t>
         </is>
       </c>
-      <c r="E132" s="31" t="inlineStr">
+      <c r="E132" s="35" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="31" t="inlineStr">
+      <c r="A133" s="35" t="inlineStr">
         <is>
           <t>2026-08-30</t>
         </is>
       </c>
-      <c r="B133" s="31" t="inlineStr">
+      <c r="B133" s="35" t="inlineStr">
         <is>
           <t>AUTO-006</t>
         </is>
       </c>
-      <c r="C133" s="31" t="inlineStr">
+      <c r="C133" s="35" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -5071,24 +5086,24 @@
           <t>Live POST to /api/auth/register with password 'ValidPass123!' and confirmPassword 'DifferentPass456!' (throwaway address shijo-regress-20260830a@mailinator.com) -&gt; HTTP 400, body {"error":"Passwords do not match"}. The server-side confirmPassword check shipped 2026-07-19 is still live and still fires ahead of any account creation. No account created. Same same-origin-fetch method as AUTO-005 (sandbox curl blocked by proxy allowlist).</t>
         </is>
       </c>
-      <c r="E133" s="31" t="inlineStr">
+      <c r="E133" s="35" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="31" t="inlineStr">
+      <c r="A134" s="35" t="inlineStr">
         <is>
           <t>2026-08-30</t>
         </is>
       </c>
-      <c r="B134" s="31" t="inlineStr">
+      <c r="B134" s="35" t="inlineStr">
         <is>
           <t>AUTO-007</t>
         </is>
       </c>
-      <c r="C134" s="31" t="inlineStr">
+      <c r="C134" s="35" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -5098,24 +5113,24 @@
           <t>Live POST to /api/auth/register with a 3-character password 'abc' in both password and confirmPassword (throwaway address shijo-regress-20260830b@mailinator.com) -&gt; HTTP 400, body {"error":"Password must be at least 8 characters"}. The 8-character minimum is enforced server-side, independent of the client form. No account created. Same same-origin-fetch method as AUTO-005.</t>
         </is>
       </c>
-      <c r="E134" s="31" t="inlineStr">
+      <c r="E134" s="35" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="31" t="inlineStr">
+      <c r="A135" s="35" t="inlineStr">
         <is>
           <t>2026-08-30</t>
         </is>
       </c>
-      <c r="B135" s="31" t="inlineStr">
+      <c r="B135" s="35" t="inlineStr">
         <is>
           <t>AUTO-008</t>
         </is>
       </c>
-      <c r="C135" s="31" t="inlineStr">
+      <c r="C135" s="35" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -5125,24 +5140,24 @@
           <t>Fetched all 16 protected routes live with credentials:'omit' and redirect:'follow', asserting the final URL landed on /login?redirect=. 16/16 passed -- every one resolved to https://www.shijo.ai/login?redirect=&lt;url-encoded original path&gt;, i.e. a real redirect with the return path preserved, never a 200 carrying authenticated UI. Route list was re-derived this run via `find app/dashboard app/admin -name page.tsx` rather than reused from the last log, which matters because the inventory CHANGED: the new untracked /dashboard/tools/geo-visibility-checker page adds a 16th route (15 last run). It was tested and correctly redirects -- note that even though it is only a redirect stub to the public /geo, middleware.ts intercepts it first, so an anonymous visitor is sent to /login rather than through to /geo. Routes covered -- dashboard: /dashboard, /ai-visibility, /analytics, /billing, /content, /keywords, /settings, /tools, /tools/keyword-research (dynamic [toolId]), /tools/geo-visibility-checker; admin: /admin, /admin/signups, /admin/terms, /admin/tickets, /admin/usage, /admin/users. Matches middleware.ts, matcher ['/dashboard/:path*','/admin/:path*']. (As logged before, app/admin/page.tsx does not exist as a file but the bare /admin path is still covered by the matcher and was verified.)</t>
         </is>
       </c>
-      <c r="E135" s="31" t="inlineStr">
+      <c r="E135" s="35" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="31" t="inlineStr">
+      <c r="A136" s="35" t="inlineStr">
         <is>
           <t>2026-08-30</t>
         </is>
       </c>
-      <c r="B136" s="31" t="inlineStr">
+      <c r="B136" s="35" t="inlineStr">
         <is>
           <t>AUTO-009</t>
         </is>
       </c>
-      <c r="C136" s="31" t="inlineStr">
+      <c r="C136" s="35" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -5152,24 +5167,24 @@
           <t>Fetched all four endpoints live with credentials:'omit', probing BOTH GET and POST on each so nothing leaks on the unintended verb. On their real method all four return 401: /api/usage GET -&gt; 401 {"error":"Not authenticated"}; /api/stripe/create-checkout POST -&gt; 401 {"error":"Please sign in first"}; /api/dashboard/ai-visibility-waitlist POST -&gt; 401 {"success":false,"error":"Please sign in to join the waitlist."}; /api/generate POST -&gt; 401 {"success":false,"error":"Please sign in to use AI tools"}. On the wrong verb each returns 405 with an empty body. No endpoint returned data and no error body disclosed anything beyond the sign-in prompt. ADDED THIS RUN: also probed the new /api/geo/scan route from the untracked GEO feature -- returns 404 on both verbs, confirming it is not deployed. When it does ship it will be a PUBLIC unauthenticated endpoint by design (it is outside the middleware matcher), so it should be added to this test as an explicit exception with its own abuse/rate-limit check rather than a 401 assertion -- lib/geo/budget.ts exists, suggesting spend control was considered, but it was not exercised here.</t>
         </is>
       </c>
-      <c r="E136" s="31" t="inlineStr">
+      <c r="E136" s="35" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="31" t="inlineStr">
+      <c r="A137" s="35" t="inlineStr">
         <is>
           <t>2026-08-30</t>
         </is>
       </c>
-      <c r="B137" s="31" t="inlineStr">
+      <c r="B137" s="35" t="inlineStr">
         <is>
           <t>AUTO-010</t>
         </is>
       </c>
-      <c r="C137" s="31" t="inlineStr">
+      <c r="C137" s="35" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -5179,24 +5194,24 @@
           <t>Read app/api/stripe/create-checkout/route.ts in full. VALID_PLANS keys are exactly {pro, growth}; 'enterprise' is absent with an inline comment recording the 2026-07-19 pause. Cross-checked against lib/stripe/products.ts rather than hardcoding the expected set: PLAN_FEATURES.enterprise carries comingSoon:true and PLAN_FEATURES.free has no priceId, so {pro, growth} is precisely the currently-purchasable set. All three guards present and correct: interval must be monthly|annual (else 400 'Invalid billing interval'); !plan || !VALID_PLANS[plan] -&gt; 400 'Invalid plan selected', catching 'enterprise' and every unrecognized name; and the interval-resolution guard !VALID_PLANS[plan][interval] -&gt; 400 'This plan is not available on that billing interval yet', correctly handling growth having monthly but no annual price. Re-verified the sibling app/api/billing/checkout/route.ts too, since it can also reach Stripe: its ALLOWED_PRICE_IDS is a hand-written list of exactly PRO_MONTHLY, PRO_ANNUAL, GROWTH_MONTHLY -- deliberately not Object.values(STRIPE_PRICE_IDS) -- so the paused ENTERPRISE_* ids are not purchasable there either. IMPORTANT CONTEXT for this whole run: local HEAD is b88b5c0 but origin/main is 48c7a84 -- THREE COMMITS ARE UNPUSHED (b88b5c0 KB update, d7b767f 'D-37 billing-month quota, hide annual, CSP report-only, D-13 atomic upsert', 0f72c97 verification pass), plus 2 modified files and 4 untracked directories. Every repo-side result in this run therefore describes local code, which is AHEAD of production. Note specifically that d7b767f hides the annual option in the UI but does NOT remove pro.annual from VALID_PLANS, so the annual price stays purchasable server-side after that ships -- intentional as far as the code reads, but worth confirming it is what was meant.</t>
         </is>
       </c>
-      <c r="E137" s="31" t="inlineStr">
+      <c r="E137" s="35" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="31" t="inlineStr">
+      <c r="A138" s="35" t="inlineStr">
         <is>
           <t>2026-08-30</t>
         </is>
       </c>
-      <c r="B138" s="31" t="inlineStr">
+      <c r="B138" s="35" t="inlineStr">
         <is>
           <t>AUTO-011</t>
         </is>
       </c>
-      <c r="C138" s="31" t="inlineStr">
+      <c r="C138" s="35" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -5206,24 +5221,24 @@
           <t>Fetched https://www.shijo.ai/sitemap.xml live -- HTTP 200, 13 &lt;loc&gt; entries, zero matches for 'dashboard' or 'admin'. Full list: /blog plus 3 blog posts (ai-seo-tools-keyword-research-faster, ai-ad-copy-that-converts, ai-marketing-tools-small-business-2026), the root, /contact, /ai-marketing-tools, and the 6 legal pages (/terms, /privacy, /cookies, /gdpr-compliance, /ai-compliance, /security). Identical to 2026-08-29. Consistent with AUTO-008: the routes middleware.ts bounces to /login are also absent from the crawlable sitemap, so there is no information-disclosure path via search. PENDING CHANGE, verified safe: app/sitemap.ts is modified locally to add ONE new public URL, https://www.shijo.ai/geo, priority 0.8. That is a genuinely public unauthenticated route, so it is not a leak -- and the diff comment explicitly records that /pricing and /features were deliberately NOT added because they 404 on production, which I confirmed live (both return 404). Re-check this test after the geo deploy: /geo itself currently 404s live, so the entry must not ship ahead of the page or the sitemap will advertise a dead URL to crawlers.</t>
         </is>
       </c>
-      <c r="E138" s="31" t="inlineStr">
+      <c r="E138" s="35" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="32" t="inlineStr">
+      <c r="A139" s="36" t="inlineStr">
         <is>
           <t>2026-08-30</t>
         </is>
       </c>
-      <c r="B139" s="32" t="inlineStr">
+      <c r="B139" s="36" t="inlineStr">
         <is>
           <t>AUTO-013</t>
         </is>
       </c>
-      <c r="C139" s="32" t="inlineStr">
+      <c r="C139" s="36" t="inlineStr">
         <is>
           <t>Fail</t>
         </is>
@@ -5233,24 +5248,24 @@
           <t>Both previously-logged violations persist, and there is a THIRD, new, unshipped one. (1) STILL LIVE in public marketing copy, now 42 days old (since commit fcd06fa, 2026-07-19): components/landing/Pricing.tsx renders '2 AI tools (Haiku-powered)' (line 27) and 'Sonnet AI for complex tasks' (lines 48 and 69). Re-confirmed live this run -- a regex sweep for /claude|anthropic|haiku|sonnet|opus/i over the rendered HTML of all three public pages returns {Haiku, Sonnet} on the homepage and NOTHING on /ai-marketing-tools or /contact. Haiku and Sonnet are Claude model names, so the homepage names the AI vendor in customer-facing copy, which the product rule confines to /privacy, /security and /ai-compliance. The compliant wording already exists in the repo -- components/lp/LandingPageContent.tsx says 'Advanced AI for complex tasks', which is exactly what /ai-marketing-tools serves live -- so the fix is to copy that phrasing into Pricing.tsx lines 27/48/69. Repeating the recommendation from the last two runs: the sheet's own Method grep ('claude|anthropic') CANNOT catch this and should be widened to 'claude|anthropic|haiku|sonnet|opus'. (2) PERSISTS, unchanged since 2026-07-20: app/gdpr-compliance/page.tsx:77 renders public text 'Anthropic -- AI model infrastructure powering platform features'. Still a policy-scope decision for Sri, not a code bug: either formally add /gdpr-compliance as a fourth approved disclosure location (defensible -- it is a legal page listing sub-processors, exactly the carve-out the rule intends) or drop the vendor name. (3) NEW, NOT YET LIVE, needs an explicit decision before the GEO feature deploys: the untracked GEO checker names Claude in customer-facing product UI. lib/geo/types.ts:42 sets ENGINE_LABELS.claude = 'Claude', which GeoChecker.tsx renders as a column header in the results grid, and app/geo/page.tsx's meta description reads '...whether ChatGPT, Gemini, Perplexity, Claude and Google AI Overviews mention your business...'. The developer anticipated this and left a rationale comment above ENGINE_LABELS arguing these labels name engines the USER asked us to query, which is a different thing from disclosing the vendor behind the 12 tools. That reasoning is sound and I am not overriding it -- but it is a new interpretation of a rule Sri wrote, so it needs Sri's explicit sign-off rather than a code comment's, especially since app/layout.tsx:14-16 documents a PRIOR incident with near-identical wording ('track your visibility in ChatGPT, Claude &amp; Perplexity') that was treated as a violation and removed on 2026-07-18. Also note lib/geo/engines/claude.ts reuses the same ANTHROPIC_API_KEY that powers the 12 dashboard tools, so the vendor genuinely is both a measured engine and the underlying supplier. Confirmed non-violations (backend or non-rendered, unchanged): app/api/generate/route.ts SDK import + model-id constants + one comment, lib/ai/claude.ts (entirely backend plumbing), lib/ai/pricing.ts model-id cost keys, lib/tools/usage.ts:50 comment, app/layout.tsx:14-16 comment, app/robots.ts:20 'Claude-Web' crawler directive, and the internal haiku/sonnet modelTier enums that ToolPage.tsx and dashboard/tools map to the neutral labels Fast/Advanced.</t>
         </is>
       </c>
-      <c r="E139" s="32" t="inlineStr">
+      <c r="E139" s="36" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
       </c>
     </row>
     <row r="140">
-      <c r="A140" s="31" t="inlineStr">
+      <c r="A140" s="35" t="inlineStr">
         <is>
           <t>2026-08-30</t>
         </is>
       </c>
-      <c r="B140" s="31" t="inlineStr">
+      <c r="B140" s="35" t="inlineStr">
         <is>
           <t>AUTO-015</t>
         </is>
       </c>
-      <c r="C140" s="31" t="inlineStr">
+      <c r="C140" s="35" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -5260,24 +5275,24 @@
           <t>Diffed programmatically: regex-extracted the tool names from buildWelcomeEmail() in lib/email.ts and from the TOOLS export in lib/tools/registry.ts, compared as sets in both directions. 12 names each side, symmetric difference empty. Exact match: Post Caption Generator, Keyword Research, SEO Content Brief, SEO Meta Generator, FAQ Generator, AI Overview Optimizer, Ad Copy Generator, Ad Headline A/B Tester, Audience Targeting Profiles, Landing Page Copy Generator, Email Sequence Generator, Newsletter Generator. (Order differs because the email groups by category -- expected, not a mismatch.) The free/paid split is also correct and was checked separately: the two tools badged FREE in the email (Post Caption Generator, SEO Meta Generator) are exactly the two registry entries with minPlan:'free'. The 24-fabricated-name regression fixed 2026-07-19 has not returned, and the hand-sync warning comment at lib/email.ts:135-139 is still in place. TWO CARRY-FORWARD NOTES: (a) the paid-tool badge TEXT in this same email is wrong ('Pro' where it should read 'Standard') -- logged under AUTO-003, not a tool-list mismatch, so it does not change this result; (b) this test is hand-synced by design, and the pending GEO checker is the next thing likely to break it -- if /geo ships and is ever mentioned in the welcome email without being added to registry.ts, this diff fails. It correctly is NOT in the email today.</t>
         </is>
       </c>
-      <c r="E140" s="31" t="inlineStr">
+      <c r="E140" s="35" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="32" t="inlineStr">
+      <c r="A141" s="36" t="inlineStr">
         <is>
           <t>2026-08-30</t>
         </is>
       </c>
-      <c r="B141" s="32" t="inlineStr">
+      <c r="B141" s="36" t="inlineStr">
         <is>
           <t>AUTO-016</t>
         </is>
       </c>
-      <c r="C141" s="32" t="inlineStr">
+      <c r="C141" s="36" t="inlineStr">
         <is>
           <t>Fail</t>
         </is>
@@ -5287,7 +5302,763 @@
           <t>One item live, two latent, one dormant, plus one NEW latent claim. (1) STILL FAILING, 5th consecutive run since 2026-08-22: components/landing/UseCases.tsx:24 renders 'Trusted by marketing teams, agencies, and brands worldwide' under a 'Built for Modern Enterprises' heading -- re-confirmed verbatim in the live homepage HTML this run, and it is the ONLY claim the live sweep surfaced across all three public pages. Unverifiable social proof (plural teams, agencies, brands, worldwide). The customer count could not be re-checked this run (AUTO-004 blocked, no DB access); the last actual reading, 2026-08-29, was 1 active subscription on Standard, which does not substantiate the wording. Needs Sri to soften the copy or confirm real customers -- not safely auto-fixable. (2) LATENT, unchanged: lib/seo-config.ts pages.features (lines 38-41) and pages.dashboard (lines 50-52) describe unbuilt capabilities as shipped -- 'clustering, intent classification, search volume checking, SERP analysis, and rank tracking', 'Enterprise-grade SEO tools', 'measuring AI search visibility', 'Real-time SEO analytics'. Both also declare canonicals pointing at /features and /dashboard; I verified live that /features returns 404, so those canonicals are dead. pages.pricing additionally still says 'Free, Pro &amp; Enterprise Plans' though Enterprise is paused, and its canonical /pricing is also a live 404. Nothing renders from these today (only pages.home is wired up) but any future generatePageMetadata('features'|'dashboard'|'pricing') call publishes fabricated claims and dead canonicals instantly. Recommend deleting the dead entries rather than leaving the trap -- note app/geo/page.tsx's own comment says the author avoided this file precisely because it is 'under an ads freeze' and its canonicals point at 404s, so the trap is now actively shaping how new code gets written. (3) STILL DORMANT: components/landing/TrustBadges.tsx retains 'SOC 2 Compliant', '99.9% Uptime', '10M+ Keywords Analyzed Daily', '500+ Enterprises'. grep across app/, components/, lib/ finds the identifier only in its own definition file -- zero imports -- and none of the four strings appear in the live HTML of any public page. Still needs a user-run rm; the sandbox cannot delete. (4) NEW, LATENT, in the untracked GEO checker: app/geo/page.tsx tells visitors 'We ask five answer engines the questions your customers actually ask' and GeoChecker.tsx's button reads 'Checking five engines...' -- both hardcode FIVE. But of the five adapters only claude.ts has its key present (ANTHROPIC_API_KEY); the local .env/.env.local contain no OPENAI_API_KEY, GEMINI_API_KEY, PERPLEXITY_API_KEY, DATAFORSEO_LOGIN/PASSWORD or GOOGLE_PLACES_API_KEY. Production env vars live in Vercel and could not be read from here, so this is NOT confirmed as a production defect -- but if those keys are absent at deploy, the page promises five engines and delivers one. Mitigating: lib/geo/orchestrator.ts degrades properly, recording unavailable engines as 'skipped' with 'Not checked -- engine unavailable' rather than scoring them as negatives, and the UI surfaces a degraded-engines notice. Recommended before shipping: confirm all five keys exist in production, or make the count dynamic from the available-adapter list instead of hardcoding 'five'. (5) CLEAN: app/layout.tsx metadata describes the real 12-tool product and claims no certifications; app/page.tsx JSON-LD omits aggregateRating and reports offerCount 3 / highPrice 199.</t>
         </is>
       </c>
-      <c r="E141" s="32" t="inlineStr">
+      <c r="E141" s="36" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="35" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B142" s="35" t="inlineStr">
+        <is>
+          <t>AUTO-001</t>
+        </is>
+      </c>
+      <c r="C142" s="35" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D142" s="22" t="inlineStr">
+        <is>
+          <t>Repo: grep -rniE '24[^0-9]{0,15}(tools|apps)' across app/, components/, lib/ returned exactly ONE hit and it is not a claim -- app/features/page.tsx:14, inside the file's header comment, recording the history ('a "24 AI tools" claim in a landing component'). Broader sweep of every '&lt;number&gt; tools/apps' phrase in source returns only 12 and 2 in use, both correct. lib/tools/registry.ts TOOLS still has exactly 12 ids and 12 names, minPlan split 2 free / 10 pro. Live: fetched /, /ai-marketing-tools, /contact AND the two brand-new public pages /pricing and /features and the now-shipped /geo (all HTTP 200). has24 regex false on all six. Count phrases across all six = {12 tools, 12 Tools, 12 AI tools, 2 tools, 2 AI tools}. MAJOR CHANGE SINCE LAST RUN, and the reason this passed rather than failed: the GEO feature flagged as the top risk on 2026-08-30 HAS NOW SHIPPED (HEAD=origin/main=83ec917, working tree clean, /geo returns 200 live where it 404'd yesterday). The '12 tools' claim survived it because the guard held exactly as designed -- the GEO checker was NOT added to lib/tools/registry.ts, /dashboard/tools/geo-visibility-checker is still only a redirect stub, and the new /features page derives its heading from TOOLS.length rather than asserting a number ({TOOLS.length} AI marketing tools, {freeCount} are free). That is the right pattern and worth copying. RESIDUAL RISK, minor: app/features/page.tsx's metadata title and description hardcode '12 AI Marketing Tools' as literal text even though the body is computed, and lib/seo-config.ts pages.features does the same -- so the page body and its own &lt;title&gt; can drift apart if a 13th tool is ever registered.</t>
+        </is>
+      </c>
+      <c r="E142" s="35" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="35" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B143" s="35" t="inlineStr">
+        <is>
+          <t>AUTO-002</t>
+        </is>
+      </c>
+      <c r="C143" s="35" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D143" s="22" t="inlineStr">
+        <is>
+          <t>Repo: grep '$99' across app/, components/, lib/ returned ZERO matches. Four bare-99 occurrences, all previously documented and all still benign: lib/stripe/products.ts:122-123 (enterprise price 99 / annualPrice 950, comingSoon:true, 'kept for reference, not currently sold'), components/landing/TrustBadges.tsx:7 '99.9% Uptime' in the still-orphaned unrendered file, app/globals.css:19 a CSS lightness value, and the two guard comments at app/page.tsx:22 and app/ai-marketing-tools/page.tsx:42 that record the retired-99 JSON-LD incident (both lines themselves read 199, so the 2026-08-23 highPrice fix still holds). NEW PRICE POINTS THIS RUN, both reconciled: a 'Plus' tier at $79/mo (PLAN_FEATURES.plus.price=79, added 2026-08-31) and a $39 one-off AI visibility report. Live: extracted every '$&lt;digits&gt;' token from six public pages. Homepage={$0,$29,$79,$278,$199}; /ai-marketing-tools={$0,$29,$199}; /contact={$29,$79,$199}; /pricing={$0,$29,$79,$199,$39}. Every figure traces to lib/stripe/products.ts via lib/pricing-plans.ts (pro 29 / annual 278, plus 79, growth 199) -- no $99 anywhere, no unexplained number. CONSISTENCY NOTE, not a price error: /ai-marketing-tools is the one ad-serving surface that still shows only $29/$199 and omits Plus entirely, so the plan lineup a visitor sees depends on which page the ad drops them on. CROSS-REFERENCE, and the more serious issue: the $79 and $39 figures are advertised with no gate on whether they can actually be bought -- see AUTO-016 item (1). The prices themselves are correct; whether a customer can pay them is not established.</t>
+        </is>
+      </c>
+      <c r="E143" s="35" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="36" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B144" s="36" t="inlineStr">
+        <is>
+          <t>AUTO-003</t>
+        </is>
+      </c>
+      <c r="C144" s="36" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="D144" s="24" t="inlineStr">
+        <is>
+          <t>CRITICAL, and unchanged for the sixth consecutive run. All three defects first logged 2026-08-22/08-29 are still present verbatim in code that is now PUSHED and live (HEAD=origin/main=83ec917, clean tree -- unlike the last five runs, these are no longer 'unpushed local' findings). (1) app/api/stripe/create-checkout/route.ts:93 still returns `You are already on the ${plan} plan`, interpolating the RAW internal key, and app/dashboard/billing/page.tsx:264-266 still renders {error} verbatim into the visible red banner. A $199 customer re-clicking upgrade is shown 'You are already on the growth plan'. One-line fix: PLAN_DISPLAY_NAME[plan]. Now 9 days old. NEWLY WORSE: 'plus' is now a valid plan key, so this same string can also emit 'you are already on the plus plan' -- lowercase, but at least not a wrong word, which makes the bug quieter without fixing it. (2) lib/email.ts:172 still badges every non-free tool with the literal string 'Pro' while all 12 tools unlock on the $29 tier displayed as 'Standard'; the same email's CTA at line 223 reads 'Unlock all 12 tools for just $29/month'. Reaches every new signup. Correct badge text is 'Standard'. (3) components/dashboard/TopBar.tsx:11 still reads 'Pro gives you 200/month across all 12 tools' -- 200/mo is Standard; Pro (growth) is 1,500. Wrong plan name AND understates Pro by 7.5x. Clean elsewhere: the only ${plan}/{userPlan}/{planTier} interpolations in app/ or components/ remain (1) plus a harmless success_url query param and a server-side console.log in webhook-handlers.ts:78. lib/stripe/plan-names.ts is intact and correctly gained 'plus' -&gt; 'Plus' with an explanatory comment. Live plan names across /, /ai-marketing-tools, /contact, /pricing are exactly {Free, Standard, Plus, Pro, Enterprise}. INVESTIGATED AND CLEARED: the live sweep flagged lowercase 'growth' on /pricing. Traced to the RSC script payload only -- a React list key ("div","growth") and the planKey:"growth" prop passed to PricingCta, whose rendered label is 'Choose Pro'. No visible text leak; the key must cross to the client because the CTA posts it to create-checkout. Not counted as a defect. Dashboard billing HTML still not diffable unauthenticated (correctly redirects), so (1),(2),(3) remain code-level verification only.</t>
+        </is>
+      </c>
+      <c r="E144" s="36" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="37" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B145" s="37" t="inlineStr">
+        <is>
+          <t>AUTO-004</t>
+        </is>
+      </c>
+      <c r="C145" s="37" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="D145" s="26" t="inlineStr">
+        <is>
+          <t>BLOCKED -- a Critical-priority test, now blocked on 6 of the last 7 runs, and its scope grew this run. No Stripe MCP connector exists in this session: ToolSearch for stripe/products/prices/billing/subscriptions returns no deferred tools, and mcp__mcp-registry__list_connectors filtered on stripe/payments/billing returns []. Fallbacks re-tested and still unavailable: the sandbox egress proxy rejects api.stripe.com at CONNECT (HTTP 403 from proxy, same as www.shijo.ai). DELIBERATELY NOT ATTEMPTED, unchanged from prior runs: STRIPE_SECRET_KEY is present in the local .env and could technically be used from the browser pane's JS context, but injecting a live secret key into a page context is a credential-exposure risk and a security-sensitive action, so it was not done unattended. Nothing was verified against Stripe this run. Still needing verification: prod_UAltLAeJGLVSqI (price_1TCQLpHTpiuftGGEZWt9UJ2Y, $29, must read 'SHIJO.AI Standard'), prod_UuvJvC2ZKysgfK (price_1Tv5SpHTpiuftGGEMu4TdOzs, $199, must read 'SHIJO.AI Pro'), prod_UAluQCvL32SQ3k (Enterprise, paused). CARRIED FORWARD, still open: the $278/yr Standard annual price is nicknamed 'Shijo Pro Annual' and the Enterprise annual price 'Shijo Enterprise Annual' -- retired branding on a price that IS still purchasable (VALID_PLANS.pro.annual) and still rendered on the live homepage. NEW SCOPE THIS RUN: two further products now need name verification and neither has a hardcoded id to check -- STRIPE_PRICE_IDS.PLUS_MONTHLY and STRIPE_PRICE_GEO_REPORT are read from the environment (a deliberate choice, documented at lib/stripe/products.ts:29-37 to avoid repeating D-39's sandbox-ids-in-a-live-constant bug). Per that same comment the LIVE-mode products for Plus and the report DO NOT EXIST YET -- only test-sandbox ones. That is unverified from here and is the single most important thing this test would settle: see AUTO-016 item (1). To unblock permanently, connect a Stripe MCP connector; it is the only way this Critical test runs unattended.</t>
+        </is>
+      </c>
+      <c r="E145" s="37" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="35" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B146" s="35" t="inlineStr">
+        <is>
+          <t>AUTO-005</t>
+        </is>
+      </c>
+      <c r="C146" s="35" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D146" s="22" t="inlineStr">
+        <is>
+          <t>Live POST to https://www.shijo.ai/api/auth/register with email 'not-a-valid-email' (name 'Regression Bot', matching valid 12-char passwords so email format was the ONLY invalid field) -&gt; HTTP 400, body {"error":"Please enter a valid email address"}. Not 200; no account created. Method: sandbox curl remains blocked by the egress proxy allowlist (403 from proxy after CONNECT on www.shijo.ai, re-confirmed this run), so the request was issued as a same-origin fetch with credentials:'omit' from a live page context in the built-in browser pane -- the identical live endpoint, and the same method used on 2026-08-23 and 2026-08-30.</t>
+        </is>
+      </c>
+      <c r="E146" s="35" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="35" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B147" s="35" t="inlineStr">
+        <is>
+          <t>AUTO-006</t>
+        </is>
+      </c>
+      <c r="C147" s="35" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D147" s="22" t="inlineStr">
+        <is>
+          <t>Live POST to /api/auth/register with password 'ValidPass123!' and confirmPassword 'DifferentPass456!' (throwaway address shijo-regress-20260831a@mailinator.com) -&gt; HTTP 400, body {"error":"Passwords do not match"}. The server-side confirmPassword check shipped 2026-07-19 is still live and still fires ahead of any account creation. No account created. Same same-origin-fetch method as AUTO-005.</t>
+        </is>
+      </c>
+      <c r="E147" s="35" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="35" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B148" s="35" t="inlineStr">
+        <is>
+          <t>AUTO-007</t>
+        </is>
+      </c>
+      <c r="C148" s="35" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D148" s="22" t="inlineStr">
+        <is>
+          <t>Live POST to /api/auth/register with a 3-character password 'abc' in both password and confirmPassword (throwaway address shijo-regress-20260831b@mailinator.com) -&gt; HTTP 400, body {"error":"Password must be at least 8 characters"}. The 8-character minimum is enforced server-side, independent of the client form. No account created. Same same-origin-fetch method as AUTO-005.</t>
+        </is>
+      </c>
+      <c r="E148" s="35" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="35" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B149" s="35" t="inlineStr">
+        <is>
+          <t>AUTO-008</t>
+        </is>
+      </c>
+      <c r="C149" s="35" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D149" s="22" t="inlineStr">
+        <is>
+          <t>18/18 passed. Route inventory was re-derived this run via `find app/dashboard app/admin -name page.tsx` rather than reused, which mattered again: the GEO deploy added TWO new admin routes since yesterday (/admin/geo-health and the dynamic /admin/geo-health/scan/[scanId]), taking the count from 16 to 18. Fetched every route live with credentials:'omit' and redirect:'follow' and asserted the final URL landed on /login?redirect=. Every one resolved to https://www.shijo.ai/login?redirect=&lt;url-encoded original path&gt; -- a real redirect preserving the return path, never a 200 carrying authenticated UI. Both new admin routes behave correctly, including the dynamic segment (tested with /admin/geo-health/scan/test123). Routes covered -- dashboard: /dashboard, /ai-visibility, /analytics, /billing, /content, /keywords, /settings, /tools, /tools/keyword-research (dynamic [toolId]), /tools/geo-visibility-checker; admin: /admin, /admin/geo-health, /admin/geo-health/scan/[scanId], /admin/signups, /admin/terms, /admin/tickets, /admin/usage, /admin/users. Matches middleware.ts matcher ['/dashboard/:path*','/admin/:path*']. As before, app/admin/page.tsx does not exist as a file but the bare /admin path is covered by the matcher and was verified.</t>
+        </is>
+      </c>
+      <c r="E149" s="35" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="35" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B150" s="35" t="inlineStr">
+        <is>
+          <t>AUTO-009</t>
+        </is>
+      </c>
+      <c r="C150" s="35" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D150" s="22" t="inlineStr">
+        <is>
+          <t>All four required endpoints return 401 unauthenticated, verified live with credentials:'omit': /api/usage GET -&gt; 401 {"error":"Not authenticated"}; /api/stripe/create-checkout POST -&gt; 401 {"error":"Please sign in first"}; /api/dashboard/ai-visibility-waitlist POST -&gt; 401 {"success":false,"error":"Please sign in to join the waitlist."}; /api/generate POST -&gt; 401 {"success":false,"error":"Please sign in to use AI tools"}. No endpoint returned data and no error body disclosed anything beyond the sign-in prompt. ADDED THIS RUN, both new with the GEO deploy: /api/admin/geo-health GET -&gt; 401 {"error":"Unauthorized"} (correct -- admin-only vendor-ping and budget data must not be readable anonymously). /api/geo/scan POST -&gt; 400 {"success":false,"error":"Please enter a business name."}, i.e. it answered an anonymous request. That is CORRECT BY DESIGN and not a failure: /geo is deliberately a public no-signup checker and the route sits outside the middleware matcher, so it validates input rather than demanding a session. It should be recorded in the Test Cases sheet as an explicit named exception to this test with its own abuse/rate-limit assertion instead of a 401 assertion -- lib/geo/budget.ts and the GEO_DAILY_BUDGET_USD / GEO_ADMIN_DAILY_SCAN_CAP env vars show spend control was designed, and the free tier is documented as 1 scan/day, but neither the per-IP limit nor the budget cap was exercised here (doing so would spend real vendor credits, which is out of scope for an unattended run).</t>
+        </is>
+      </c>
+      <c r="E150" s="35" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="35" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B151" s="35" t="inlineStr">
+        <is>
+          <t>AUTO-010</t>
+        </is>
+      </c>
+      <c r="C151" s="35" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D151" s="22" t="inlineStr">
+        <is>
+          <t>Read app/api/stripe/create-checkout/route.ts in full. VALID_PLANS is declared with exactly {pro, growth}; 'enterprise' is absent with the inline comment recording the 2026-07-19 pause. Cross-checked against lib/stripe/products.ts rather than hardcoding the expected set: PLAN_FEATURES.enterprise carries comingSoon:true and PLAN_FEATURES.free has no priceId, so the paid self-serve set is {pro, growth} plus the new conditional 'plus'. All three guards present and correct: interval must be monthly|annual (else 400 'Invalid billing interval'); !plan || !VALID_PLANS[plan] -&gt; 400 'Invalid plan selected', catching 'enterprise' and every unrecognized name; and the interval-resolution guard !VALID_PLANS[plan][interval] -&gt; 400, correctly handling growth having monthly but no annual price. NEW THIS RUN and the reason this still passes: 'plus' is registered CONDITIONALLY at module scope -- `if (STRIPE_PRICE_IDS.PLUS_MONTHLY) VALID_PLANS.plus = {...}` -- so on an environment where the price id is unset, Plus is simply not purchasable and falls through to the same 'Invalid plan selected' 400 rather than reaching Stripe with an empty price id. Server-side enforcement is exactly right. What is NOT right is that no UI surface consults the same condition -- see AUTO-016 item (1). Re-verified the sibling app/api/billing/checkout/route.ts: its ALLOWED_PRICE_IDS is still a hand-written list of exactly PRO_MONTHLY, PRO_ANNUAL, GROWTH_MONTHLY (deliberately not Object.values(STRIPE_PRICE_IDS)), so the paused ENTERPRISE_* ids are not purchasable there either -- note it has NOT been extended for Plus, so that route cannot sell Plus at all. REPO STATE, materially different from the last five runs: HEAD == origin/main == 83ec917, working tree completely clean, zero unpushed commits and zero untracked files. Every repo-side result in this run therefore describes code that is actually deployed, not a local tree ahead of production.</t>
+        </is>
+      </c>
+      <c r="E151" s="35" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="35" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B152" s="35" t="inlineStr">
+        <is>
+          <t>AUTO-011</t>
+        </is>
+      </c>
+      <c r="C152" s="35" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D152" s="22" t="inlineStr">
+        <is>
+          <t>Fetched https://www.shijo.ai/sitemap.xml live -- HTTP 200, 16 &lt;loc&gt; entries, zero matches for 'dashboard' or 'admin'. Grew from 13 to 16 with the GEO deploy: /pricing, /features and /geo were added. All three were verified live at HTTP 200 this run, so the concern raised on 2026-08-30 (that the /geo sitemap entry might ship ahead of the page and advertise a dead URL) did NOT materialise -- and the /pricing and /features canonicals declared in lib/seo-config.ts, which pointed at 404s for weeks, now resolve. Full list: /blog plus 3 blog posts, the root, /pricing, /features, /geo, the 6 legal pages (/terms, /privacy, /cookies, /gdpr-compliance, /ai-compliance, /security), /contact and /ai-marketing-tools. Consistent with AUTO-008: every route middleware.ts bounces to /login is absent from the crawlable sitemap, including the two new /admin/geo-health routes, so there is no information-disclosure path via search.</t>
+        </is>
+      </c>
+      <c r="E152" s="35" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="36" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B153" s="36" t="inlineStr">
+        <is>
+          <t>AUTO-013</t>
+        </is>
+      </c>
+      <c r="C153" s="36" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="D153" s="24" t="inlineStr">
+        <is>
+          <t>One long-standing violation FIXED, one persists, and the violation flagged as 'not yet live, needs a decision' on 2026-08-30 HAS NOW SHIPPED TO PRODUCTION without that decision being recorded. (1) FIXED -- the 42-day-old homepage violation is gone. components/landing/Pricing.tsx no longer says '2 AI tools (Haiku-powered)' or 'Sonnet AI for complex tasks'; it now reads '2 AI tools included' and 'Advanced AI for complex tasks', matching the compliant wording that components/lp/LandingPageContent.tsx already used. Verified live: a /claude|anthropic|haiku|sonnet|opus/i sweep over the rendered HTML of /, /ai-marketing-tools and /contact now returns NOTHING on all three. (2) NOW LIVE, was flagged as pending last run: the GEO feature names Claude in customer-facing surfaces on production. app/features/page.tsx:84 hardcodes an engine list ['ChatGPT Search','Google Gemini','Perplexity','Claude','Google AI Overviews'] rendered as visible &lt;li&gt; bullets -- confirmed in the live /features HTML as '...&gt;Claude&lt;/li&gt;'. app/geo/page.tsx:23's meta description reads '...whether ChatGPT, Gemini, Perplexity, Claude and Google AI Overviews mention your business...' -- confirmed in the live /geo &lt;meta name="description"&gt;, so it is also what search engines and social scrapers will quote. The developer's rationale (naming engines the USER asked us to query is not the same as disclosing the vendor behind the 12 tools) is recorded in a code comment above ENGINE_LABELS in lib/geo/types.ts and is a defensible reading -- but it is a NEW interpretation of a rule Sri wrote, it shipped on a code comment's authority rather than Sri's, and app/layout.tsx:14-16 documents a PRIOR incident with near-identical wording ('track your visibility in ChatGPT, Claude &amp; Perplexity') that was treated as a violation and removed on 2026-07-18. Note also that app/features/page.tsx hardcodes the list rather than importing ENGINE_LABELS, so the rationale comment is not even attached to the copy that is live. This needs an explicit yes/no from Sri; until then this test cannot pass. (3) PERSISTS, unchanged since 2026-07-20: app/gdpr-compliance/page.tsx:77 renders public text 'Anthropic -- AI model infrastructure powering platform features'. Still a policy-scope decision, not a code bug: either formally add /gdpr-compliance as a fourth approved disclosure location (defensible -- it is a legal page listing sub-processors) or drop the vendor name. Confirmed non-violations (backend, admin-only or comments): app/api/generate/route.ts SDK import and model-id constants, lib/ai/claude.ts and lib/ai/pricing.ts, lib/geo/engines/claude.ts, app/layout.tsx:14-16 and lib/tools/usage.ts:50 comments, app/robots.ts:20 'Claude-Web' crawler directive, and app/admin/geo-health/GeoHealthClient.tsx:181 plus app/api/admin/geo-health/route.ts:19 (both behind the admin auth verified in AUTO-009, not customer-facing). METHOD NOTE, repeated for the third run: the sheet's Method grep ('claude|anthropic') would have MISSED the Haiku/Sonnet violation entirely -- widen it to 'claude|anthropic|haiku|sonnet|opus'.</t>
+        </is>
+      </c>
+      <c r="E153" s="36" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="35" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B154" s="35" t="inlineStr">
+        <is>
+          <t>AUTO-015</t>
+        </is>
+      </c>
+      <c r="C154" s="35" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D154" s="22" t="inlineStr">
+        <is>
+          <t>Diffed programmatically: regex-extracted the tool names from buildWelcomeEmail() in lib/email.ts and from the TOOLS export in lib/tools/registry.ts, compared as sets in both directions. 12 names each side, symmetric difference empty in both directions. Exact match: Post Caption Generator, Keyword Research, SEO Content Brief, SEO Meta Generator, FAQ Generator, AI Overview Optimizer, Ad Copy Generator, Ad Headline A/B Tester, Audience Targeting Profiles, Landing Page Copy Generator, Email Sequence Generator, Newsletter Generator. (Order differs because the email groups by category -- expected.) The free/paid split was checked separately and is correct: the two tools badged FREE in the email (Post Caption Generator, SEO Meta Generator) are exactly the two registry entries with minPlan:'free'. The 24-fabricated-name regression fixed 2026-07-19 has not returned and the hand-sync warning comment at lib/email.ts:135-139 is still in place. Specifically re-checked after the GEO deploy, since that was flagged last run as the likeliest thing to break this diff: the welcome email does NOT mention the GEO checker, /geo or AI visibility at all, so the 12-for-12 match holds. CARRY-FORWARD: the paid-tool badge TEXT in this same email is still wrong ('Pro' where it should read 'Standard') -- that is AUTO-003 defect (2), not a tool-list mismatch, so it does not change this result. Also note the email's CTA still says '$29/month' and makes no mention of the new Plus tier, which is correct today but is the next thing likely to drift.</t>
+        </is>
+      </c>
+      <c r="E154" s="35" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="36" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B155" s="36" t="inlineStr">
+        <is>
+          <t>AUTO-016</t>
+        </is>
+      </c>
+      <c r="C155" s="36" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="D155" s="24" t="inlineStr">
+        <is>
+          <t>Two items fixed, one NEW and higher-severity, two persisting. (1) NEW, HIGH SEVERITY, and the most important finding of this run: the live site advertises two products with no check that either can actually be bought. lib/stripe/products.ts defines isPlusPurchasable() and isReportPurchasable() precisely for this, with a comment explaining that PLUS_MONTHLY and GEO_REPORT are env-driven because the LIVE-mode Stripe products DO NOT EXIST YET (test sandbox only). Both functions are DEAD CODE -- grep across app/, components/, lib/ and scripts/ finds zero callers. Consequences: /pricing renders the Plus card at $79 with an active 'Choose Plus' PricingCta that POSTs planKey 'plus' to create-checkout, and the homepage and /contact also show $79 -- but create-checkout only registers VALID_PLANS.plus `if (STRIPE_PRICE_IDS.PLUS_MONTHLY)`, so if STRIPE_PRICE_PLUS_MONTHLY is unset in Vercel production, every signed-in customer clicking Choose Plus gets a 400 'Invalid plan selected', and a signed-out one is sent through /register?plan=plus to the same dead end. Separately app/api/billing/checkout/route.ts's ALLOWED_PRICE_IDS was never extended for Plus, so that route cannot sell it either. The $39 'One-off Report' card is milder -- cta is null so the button renders 'Coming soon' -- but its features still render with Check ticks rather than the Minus used for comingSoon plans, and the /pricing meta description (and lib/seo-config.ts pages.pricing) advertises 'One-off AI visibility report $39' with no such qualifier, so that is what a search result will say about a product that cannot be purchased. NOT CONFIRMED AS A PRODUCTION DEFECT -- the Vercel env cannot be read from here and AUTO-004 is blocked, so whether STRIPE_PRICE_PLUS_MONTHLY is set live is unknown. Sri should check that env var first; if it is unset, this is a live broken paid funnel on a page ads point at. The fix either way is to gate the Plus card and CTA on isPlusPurchasable() and the report card on isReportPurchasable(), which is what those functions were written for. (2) NEW, MINOR: app/page.tsx JSON-LD is now stale -- offerCount is still '3' with a comment reading 'Free, Standard and Pro are purchasable', but Plus makes four advertised plans. highPrice '199' is still correct. (3) STILL FAILING, 6th consecutive run since 2026-08-22: components/landing/UseCases.tsx:24 renders 'Trusted by marketing teams, agencies, and brands worldwide' under a 'Built for Modern Enterprises' heading -- re-confirmed verbatim in the live homepage HTML. Unverifiable social proof (plural teams, agencies, brands, worldwide); the last actual customer reading, 2026-08-29, was 1 active subscription. Not safely auto-fixable -- needs Sri to soften the copy. (4) STILL DORMANT: components/landing/TrustBadges.tsx retains 'SOC 2 Compliant', '99.9% Uptime', '10M+ Keywords Analyzed Daily', '500+ Enterprises'. Zero imports anywhere and none of the four strings appear in any live page. Still needs a user-run rm; the sandbox cannot delete. (5) FIXED: lib/seo-config.ts pages.features and pages.pricing were rewritten on 2026-08-31 and no longer describe unbuilt capabilities (clustering, intent classification, SERP analysis, rank tracking) or declare canonicals for 404s -- /features and /pricing now both return 200 and the descriptions match what those pages actually contain. seoConfig.organization.logo also now points at a real asset. (6) STILL LATENT, the last of the dead-config traps: pages.dashboard survives untouched and still promises 'monitoring rankings, analyzing SERP performance, and measuring AI search visibility. Real-time SEO analytics' with a canonical at /dashboard, an auth-gated route that must never be a canonical target. Nothing renders it today (only home, and now features/pricing via their own metadata exports), but one generatePageMetadata('dashboard') call publishes it. Recommend deleting the entry. (7) UNRESOLVED FROM LAST RUN, now live: /features says 'We ask five answer engines', /pricing says 'A single full scan across five answer engines' and the GEO UI hardcodes five. Only one of the five adapter keys (ANTHROPIC_API_KEY) is present locally; OPENAI_API_KEY, GEMINI_API_KEY, PERPLEXITY_API_KEY, DATAFORSEO_LOGIN/PASSWORD and GOOGLE_PLACES_API_KEY are absent from .env and .env.local. Production env is in Vercel and unreadable from here, and running a live scan to find out would spend real vendor credits, so this is still NOT confirmed as a production defect. Mitigating: lib/geo/orchestrator.ts degrades properly, recording unavailable engines as 'skipped' rather than scoring them as negatives, and the UI shows a degraded-engines notice. Before further ad spend on /geo, confirm all five keys exist in production or make the count dynamic.</t>
+        </is>
+      </c>
+      <c r="E155" s="36" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B156" s="10" t="inlineStr">
+        <is>
+          <t>AUTO-001</t>
+        </is>
+      </c>
+      <c r="C156" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D156" s="11" t="inlineStr">
+        <is>
+          <t>Repo: grep -rniE '24[^0-9]{0,15}(tools|apps)' across app/, components/, lib/ returned exactly ONE hit and it is not a claim -- app/features/page.tsx:14, inside the file's header comment recording the history ('a "24 AI tools" claim in a landing component'). Identical to the last run. Broader sweep of every '&lt;number&gt; tools/apps' phrase in source returns only {12 tools x39, 2 tools x21, 12 AI tools x9, 2 AI tools x4, 12 Tools x4} -- all correct. lib/tools/registry.ts TOOLS parsed programmatically: exactly 12 ids and 12 names, minPlan split 2 free / 10 pro. Live: fetched /, /ai-marketing-tools, /contact plus /pricing, /features and /geo (all HTTP 200). The 24-regex is false on all six. Count phrases across all six = {12 tools, 12 Tools, 12 AI tools, 2 tools, 2 AI tools}. Nothing regressed and no new numeric claim appeared. RESIDUAL RISK, unchanged and worth fixing when convenient: app/features/page.tsx's metadata title/description and lib/seo-config.ts pages.features both hardcode '12 AI marketing tools' as literal text while the page BODY derives its heading from TOOLS.length -- so the rendered body and the page's own &lt;title&gt; can silently drift apart if a 13th tool is ever registered. The TOOLS.length pattern used in the body is the right one and should be copied into the metadata.</t>
+        </is>
+      </c>
+      <c r="E156" s="10" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B157" s="10" t="inlineStr">
+        <is>
+          <t>AUTO-002</t>
+        </is>
+      </c>
+      <c r="C157" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D157" s="11" t="inlineStr">
+        <is>
+          <t>Repo: grep '$99' across app/, components/, lib/ returned ZERO matches. The four bare-99 occurrences are all previously documented and still benign: lib/stripe/products.ts:122-123 (enterprise price 99 / annualPrice 950, comingSoon:true, 'kept for reference, not currently sold'), components/landing/TrustBadges.tsx:7 '99.9% Uptime' in the still-orphaned unrendered file, app/globals.css:19 a CSS lightness value, and the two guard comments at app/page.tsx:22 and app/ai-marketing-tools/page.tsx:42 recording the retired-99 JSON-LD incident (both those lines themselves read 199, so the 2026-08-23 highPrice fix still holds). Source $-token census: $199 x23, $29 x22, $79 x12, $0 x5, $278 x3, $39 x2, and singletons $97/$36/$10/$3/$2/$1 -- every singleton traced and benign ($97 is placeholder copy in registry.ts:196, $36 a proration example in a webhook-handlers comment, $10 a vendor-cost note, $3/$2/$1 are regex backreferences in lib/tools/output.ts and 'less than $1 a day' upgrade copy). Live: extracted every $&lt;digits&gt; token from six public pages and resolved each in context. Homepage={$0,$29,$278,$79,$199}; /ai-marketing-tools={$0,$29,$199}; /contact={$29,$79,$199}; /pricing={$0,$29,$79,$199,$39}. Every figure traces to lib/stripe/products.ts via lib/pricing-plans.ts (pro 29 / annual 278, plus 79, growth 199, report 39). NEW METHOD NOTE for future runs: a naive $-regex on the live HTML also returns $1,$10,$14,$16,$17,$19,$20,$22 -- these are NOT prices, they are Next.js RSC payload reference markers inside self.__next_f.push scripts. Each was checked in context this run; strip &lt;script&gt; tags before the price sweep or they will produce false alarms. No $99 anywhere. CONSISTENCY NOTE, not a price error and unchanged from last run: /ai-marketing-tools -- the ad-serving surface -- still shows only Free/$29/$199 and omits Plus entirely, so the plan lineup a visitor sees still depends on which page an ad drops them on.</t>
+        </is>
+      </c>
+      <c r="E157" s="10" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B158" s="7" t="inlineStr">
+        <is>
+          <t>AUTO-003</t>
+        </is>
+      </c>
+      <c r="C158" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="D158" s="6" t="inlineStr">
+        <is>
+          <t>CRITICAL, and unchanged for the SEVENTH consecutive run. All three defects first logged 2026-08-22/08-29 are still present verbatim, still on pushed-and-live code (HEAD == origin/main == 20d3c7b; the only uncommitted files are .gitignore, SHIJO_AI_KB.md, this workbook and four untracked docs). (1) app/api/stripe/create-checkout/route.ts:93 still returns `You are already on the ${plan} plan`, interpolating the RAW internal key, and it is now duplicated at line 211 inside the new subscriber-guard/billing-portal branch -- so there are TWO sites emitting it, up from one. app/dashboard/billing/page.tsx:266 still renders {error} verbatim into the visible red banner. A $199 customer re-clicking upgrade is shown 'You are already on the growth plan'; a Plus customer gets 'the plus plan'. One-line fix at both sites: PLAN_DISPLAY_NAME[plan]. Now 10 days old. (2) lib/email.ts:172 still badges every non-free tool with the literal string 'Pro' while all 12 tools unlock on the $29 tier displayed as 'Standard'; the same email's CTA at line 223 reads 'Unlock all 12 tools for just $29/month'. Reaches every new signup. Correct badge text is 'Standard'. (3) components/dashboard/TopBar.tsx:11 still reads 'Pro gives you 200/month across all 12 tools' -- 200/mo is Standard; Pro (growth) is 1,500. Wrong plan name AND understates Pro by 7.5x. Clean elsewhere: the only ${plan}/{userPlan}/{planTier} interpolations remaining in app/ or components/ are the two at (1), three harmless success_url/cancel_url/return_url query params, a /login?plan= link in RegisterSignInLink.tsx, and two server-side console.logs in webhook-handlers.ts. lib/stripe/plan-names.ts is intact with free/pro-&gt;Standard/plus-&gt;Plus/growth-&gt;Pro/enterprise. LIVE CHECK, all clean this run: plan-card headings extracted from the rendered DOM (leaf elements only, scripts stripped) are exactly {Free, Standard, Plus, Pro, Enterprise} on /, /pricing and /ai-marketing-tools, and /contact's bullet list matches. Zero raw internal keys in visible text on any public page. The lowercase 'growth'/'plus'/'pro' strings still present in the /pricing raw HTML are confined to the RSC script payload (React list keys and the planKey prop PricingCta posts to create-checkout) -- re-confirmed, not a visible leak, not counted. One false positive investigated and cleared: the homepage heading 'Choose Your Growth Plan' is marketing copy, not the 'growth' tier key. Dashboard billing HTML still not diffable unauthenticated (it correctly 30x's to /login -- see AUTO-008), so (1),(2),(3) remain code-level verification only.</t>
+        </is>
+      </c>
+      <c r="E158" s="7" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="38" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B159" s="38" t="inlineStr">
+        <is>
+          <t>AUTO-004</t>
+        </is>
+      </c>
+      <c r="C159" s="38" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="D159" s="39" t="inlineStr">
+        <is>
+          <t>BLOCKED -- a Critical-priority test, now blocked on 7 of the last 8 runs. No Stripe MCP connector exists in this session: ToolSearch for 'stripe products prices subscriptions billing' returns no deferred tools, and mcp__mcp-registry__list_connectors filtered on stripe/payments/billing returns []. Fallbacks re-tested and still unavailable: the sandbox egress proxy rejects api.stripe.com at CONNECT (HTTP 403 from proxy, identical to www.shijo.ai). DELIBERATELY NOT ATTEMPTED, unchanged from prior runs: STRIPE_SECRET_KEY is present in the local .env and could technically be used from the browser pane's JS context, but injecting a live secret key into a page context is a credential-exposure risk and a security-sensitive action, so it was not done in an unattended run. Nothing was verified against Stripe this run. Still needing verification: prod_UAltLAeJGLVSqI (price_1TCQLpHTpiuftGGEZWt9UJ2Y, $29, must read 'SHIJO.AI Standard'), prod_UuvJvC2ZKysgfK (price_1Tv5SpHTpiuftGGEMu4TdOzs, $199, must read 'SHIJO.AI Pro'), prod_UAluQCvL32SQ3k (Enterprise, paused). CARRIED FORWARD, still open: the $278/yr Standard annual price (price_1TuEaIHTpiuftGGEslehCB4Y) is nicknamed 'Shijo Pro Annual' -- retired branding on a price that IS still purchasable via VALID_PLANS.pro.annual and is still rendered on the live homepage as '$278/year'. ALSO STILL UNVERIFIABLE, and this run's most consequential unknown: STRIPE_PRICE_IDS.PLUS_MONTHLY and STRIPE_PRICE_GEO_REPORT are read from the environment by design (lib/stripe/products.ts:29-37) and are ABSENT from the local .env/.env.local. Whether they are set in Vercel production cannot be determined from here -- /api/stripe/create-checkout returns 401 before it ever evaluates the plan, so there is no unauthenticated probe that settles it. That single env var decides whether the live 'Choose Plus' button works or dead-ends -- see AUTO-016 item (1). To unblock permanently, connect a Stripe MCP connector; it remains the only way this Critical test runs unattended.</t>
+        </is>
+      </c>
+      <c r="E159" s="38" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B160" s="10" t="inlineStr">
+        <is>
+          <t>AUTO-005</t>
+        </is>
+      </c>
+      <c r="C160" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D160" s="11" t="inlineStr">
+        <is>
+          <t>Live POST to https://www.shijo.ai/api/auth/register with email 'not-a-valid-email' (name 'Regression Bot', matching valid 13-char passwords so email format was the ONLY invalid field) -&gt; HTTP 400, body {"error":"Please enter a valid email address"}. Not 200; no account created. Method: sandbox curl remains blocked by the egress proxy allowlist (403 from proxy after CONNECT on www.shijo.ai, re-confirmed this run), so the request was issued as a same-origin fetch with credentials:'omit' from a live page context in the built-in browser pane -- the identical live endpoint, and the same method used on 2026-08-23, 08-30 and 08-31.</t>
+        </is>
+      </c>
+      <c r="E160" s="10" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B161" s="10" t="inlineStr">
+        <is>
+          <t>AUTO-006</t>
+        </is>
+      </c>
+      <c r="C161" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D161" s="11" t="inlineStr">
+        <is>
+          <t>Live POST to /api/auth/register with password 'ValidPass123!' and confirmPassword 'DifferentPass456!' (throwaway address shijo-regress-20260901a@mailinator.com) -&gt; HTTP 400, body {"error":"Passwords do not match"}. The server-side confirmPassword check shipped 2026-07-19 is still live and still fires ahead of any account creation. No account created. Same same-origin-fetch method as AUTO-005.</t>
+        </is>
+      </c>
+      <c r="E161" s="10" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B162" s="10" t="inlineStr">
+        <is>
+          <t>AUTO-007</t>
+        </is>
+      </c>
+      <c r="C162" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D162" s="11" t="inlineStr">
+        <is>
+          <t>Live POST to /api/auth/register with a 3-character password 'abc' in both password and confirmPassword (throwaway address shijo-regress-20260901b@mailinator.com) -&gt; HTTP 400, body {"error":"Password must be at least 8 characters"}. The 8-character minimum is enforced server-side, independent of the client form. No account created. Same same-origin-fetch method as AUTO-005.</t>
+        </is>
+      </c>
+      <c r="E162" s="10" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B163" s="10" t="inlineStr">
+        <is>
+          <t>AUTO-008</t>
+        </is>
+      </c>
+      <c r="C163" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D163" s="11" t="inlineStr">
+        <is>
+          <t>17/17 passed. Route inventory was re-derived this run rather than reused (find app/dashboard app/admin -name page.tsx), giving 16 static routes; the dynamic /admin/geo-health/scan/[scanId] was additionally exercised with a dummy id, and /dashboard/tools/[toolId] with a real tool id (post-caption-generator). Every one of the 17 was fetched twice with credentials:'omit': first with redirect:'manual', which returned an opaqueredirect on all 17 (i.e. a real 30x, never a 200 with content), then with redirect:'follow', which landed all 17 on https://www.shijo.ai/login?redirect=&lt;the original path, url-encoded&gt;. Response bodies were byte-identical across all 17 (14,986 chars each), confirming they render the same login shell and not per-route authenticated UI. Routes covered: /admin/{geo-health, geo-health/scan/test123, signups, terms, tickets, usage, users} and /dashboard/{'', ai-visibility, analytics, billing, content, keywords, settings, tools, tools/post-caption-generator, tools/geo-visibility-checker}. No leakage of any authenticated markup.</t>
+        </is>
+      </c>
+      <c r="E163" s="10" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B164" s="10" t="inlineStr">
+        <is>
+          <t>AUTO-009</t>
+        </is>
+      </c>
+      <c r="C164" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D164" s="11" t="inlineStr">
+        <is>
+          <t>All four required endpoints return 401 unauthenticated, verified live with credentials:'omit' from the browser pane: /api/usage GET -&gt; 401 {"error":"Not authenticated"}; /api/stripe/create-checkout POST {plan:'pro',interval:'monthly'} -&gt; 401 {"error":"Please sign in first"}; /api/dashboard/ai-visibility-waitlist POST -&gt; 401 {"success":false,"error":"Please sign in to join the waitlist."}; /api/generate POST -&gt; 401 {"success":false,"error":"Please sign in to use AI tools"}. Note for AUTO-004/016 cross-reference: create-checkout's auth guard fires BEFORE plan validation, which is correct security design but means an unauthenticated probe cannot be used to discover whether the 'plus' plan is registered in production.</t>
+        </is>
+      </c>
+      <c r="E164" s="10" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B165" s="10" t="inlineStr">
+        <is>
+          <t>AUTO-010</t>
+        </is>
+      </c>
+      <c r="C165" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D165" s="11" t="inlineStr">
+        <is>
+          <t>Read app/api/stripe/create-checkout/route.ts in full and reconciled against lib/stripe/products.ts rather than against a hardcoded expectation. VALID_PLANS is declared with exactly {pro, growth}; 'enterprise' is absent, matching PLAN_FEATURES.enterprise.comingSoon === true in products.ts, with an inline comment explaining the 2026-07-19 pause. 'plus' is added conditionally at line 36 -- `if (STRIPE_PRICE_IDS.PLUS_MONTHLY) VALID_PLANS.plus = {...}` -- which is the correct gate: PLUS_MONTHLY is env-driven and empty-string when unset, so an environment without the price id simply cannot sell Plus and falls through to the existing 'Invalid plan selected' 400. Both guards present and ordered correctly: the interval guard rejects anything other than monthly/annual (400 'Invalid billing interval') BEFORE the plan lookup, then !VALID_PLANS[plan] -&gt; 400 'Invalid plan selected', then the per-interval resolution check -&gt; 400 'This plan is not available on that billing interval yet' (this is what protects 'growth', which has no annual price). A second identical priceId null-check sits at line 133 as a belt-and-braces guard. The server-side enforcement is sound and independent of the UI. CROSS-REFERENCE, not a defect of this test: the very gate that makes this pass is the reason the Plus card can dead-end -- /pricing advertises Plus unconditionally while checkout registers it conditionally. That mismatch is logged under AUTO-016, not here.</t>
+        </is>
+      </c>
+      <c r="E165" s="10" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B166" s="10" t="inlineStr">
+        <is>
+          <t>AUTO-011</t>
+        </is>
+      </c>
+      <c r="C166" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D166" s="11" t="inlineStr">
+        <is>
+          <t>Fetched https://www.shijo.ai/sitemap.xml live -- HTTP 200, 16 &lt;loc&gt; entries, zero matches for 'dashboard' or 'admin' (case-insensitive) anywhere in the document. Unchanged from last run at 16 entries: /blog plus 3 blog posts, the apex, /pricing, /features, /geo, /terms, /privacy, /cookies, /gdpr-compliance, /ai-compliance, /security, /contact, /ai-marketing-tools. All use the canonical www host. Also re-checked /robots.txt (HTTP 200) as a defence-in-depth companion: Disallow /api/, /admin/ and /dashboard/ are all present under User-Agent: *, and the four AI-crawler allowances (GPTBot, ChatGPT-User, Claude-Web, PerplexityBot) plus the Sitemap directive are intact.</t>
+        </is>
+      </c>
+      <c r="E166" s="10" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B167" s="7" t="inlineStr">
+        <is>
+          <t>AUTO-013</t>
+        </is>
+      </c>
+      <c r="C167" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="D167" s="6" t="inlineStr">
+        <is>
+          <t>Unchanged from last run -- the two live violations flagged on 2026-08-31 are still in production and still awaiting Sri's decision, which has not been recorded anywhere in the repo. (1) NAMED IN CUSTOMER-FACING COPY, live: app/features/page.tsx:84 hardcodes 'Claude' in a rendered engine-list bullet, and app/geo/page.tsx:23's meta description reads '...whether ChatGPT, Gemini, Perplexity, Claude and Google AI Overviews mention your business...'. A /claude|anthropic|haiku|sonnet|opus/i sweep over the LIVE rendered HTML confirms 'Claude' present on /features and /geo, and confirms it is ABSENT from /, /ai-marketing-tools, /contact and /pricing. Because it sits in a meta description, the /geo instance is also what search engines and social scrapers will quote. The developer's rationale (naming the engines a USER asked us to query is not the same as disclosing the vendor behind the 12 tools) is recorded in a code comment above ENGINE_LABELS in lib/geo/types.ts and is defensible -- but it is a NEW interpretation of a rule Sri wrote, it shipped on a code comment's authority rather than Sri's, and app/layout.tsx:14-16 documents a PRIOR incident with near-identical wording ('track your visibility in ChatGPT, Claude &amp; Perplexity') that was treated as a violation and removed on 2026-07-18. app/features/page.tsx also hardcodes the list instead of importing ENGINE_LABELS, so the rationale comment is not even attached to the copy that is live. Until Sri gives an explicit yes/no this test cannot pass. (2) PERSISTS, unchanged since 2026-07-20: app/gdpr-compliance/page.tsx:77 renders public text 'Anthropic -- AI model infrastructure powering platform features'. Still a policy-scope decision, not a code bug: either formally add /gdpr-compliance as a fourth approved disclosure location (defensible -- it is a legal page listing sub-processors, and it sits alongside /privacy, /security and /ai-compliance in the footer) or drop the vendor name. (3) STILL FIXED, no regression: components/landing/Pricing.tsx remains free of the 'Haiku-powered'/'Sonnet AI' wording removed on 2026-08-31, and the homepage, /ai-marketing-tools and /contact are clean on the widened regex. Confirmed non-violations (backend, admin-only, or comments): app/api/generate/route.ts SDK import and model-id constants, lib/ai/claude.ts, lib/ai/pricing.ts, lib/geo/engines/claude.ts, lib/geo/health.ts, lib/geo/orchestrator.ts, lib/geo/types.ts, lib/geo/scoring.ts, lib/stripe/products.ts and lib/tools/usage.ts comments, app/layout.tsx:14-16 comment, app/robots.ts:20 'Claude-Web' crawler directive, app/dashboard/tools/page.tsx + components/dashboard/ToolPage.tsx (which correctly render 'Fast'/'Advanced AI' to users and keep haiku/sonnet as internal identifiers only), and app/admin/geo-health/* plus app/api/admin/geo-health/route.ts (behind the admin auth verified in AUTO-008). METHOD NOTE, repeated for the fourth run: the sheet's Method column still says grep 'claude|anthropic', which would have MISSED the Haiku/Sonnet class of violation entirely -- please widen the recorded method to 'claude|anthropic|haiku|sonnet|opus'.</t>
+        </is>
+      </c>
+      <c r="E167" s="7" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B168" s="10" t="inlineStr">
+        <is>
+          <t>AUTO-015</t>
+        </is>
+      </c>
+      <c r="C168" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D168" s="11" t="inlineStr">
+        <is>
+          <t>Diffed programmatically: regex-extracted the tool names from buildWelcomeEmail() in lib/email.ts and from the TOOLS export in lib/tools/registry.ts, compared as sets in both directions. 12 names each side, symmetric difference empty. Exact match: Post Caption Generator, Keyword Research, SEO Content Brief, SEO Meta Generator, FAQ Generator, AI Overview Optimizer, Ad Copy Generator, Ad Headline A/B Tester, Audience Targeting Profiles, Landing Page Copy Generator, Email Sequence Generator, Newsletter Generator. (Order differs because the email groups by category -- expected, not a mismatch.) The free/paid split was checked separately and is also correct: the two tools badged FREE in the email (Post Caption Generator, SEO Meta Generator) are exactly the two registry entries with minPlan:'free'. The 24-fabricated-name regression fixed 2026-07-19 has not returned. TWO CARRY-FORWARD NOTES, both unchanged: (a) the paid-tool badge TEXT in this same email is wrong ('Pro' where it should read 'Standard') -- logged under AUTO-003, not a tool-list mismatch, so it does not change this result; (b) this list is hand-synced by design and the GEO checker remains the most likely thing to break it -- /geo is live and sold on /pricing but is correctly still ABSENT from both registry.ts and the welcome email, so the diff holds.</t>
+        </is>
+      </c>
+      <c r="E168" s="10" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B169" s="7" t="inlineStr">
+        <is>
+          <t>AUTO-016</t>
+        </is>
+      </c>
+      <c r="C169" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="D169" s="6" t="inlineStr">
+        <is>
+          <t>Four items, no change in severity from last run: the highest-severity finding is still unresolved and still unverifiable from here. (1) STILL FAILING, HIGH SEVERITY, unchanged since 2026-08-31 -- the live site sells a product with no check that it can be bought. lib/stripe/products.ts:182-186 defines isPlusPurchasable() and isReportPurchasable() for exactly this purpose, with a comment explaining that PLUS_MONTHLY and GEO_REPORT are env-driven because the LIVE-mode Stripe products do not exist yet. Both functions are STILL DEAD CODE -- grep across app/, components/, lib/ and scripts/ finds zero callers, only the definitions and the comment that mentions them. Re-confirmed live this run by reading the rendered /pricing DOM: the Plus card shows $79 with an ACTIVE &lt;button&gt;Choose Plus&lt;/button&gt; (not a disabled or 'Coming soon' state), sitting alongside Choose Standard and Choose Pro, and the homepage and /contact also advertise $79. But create-checkout registers VALID_PLANS.plus only `if (STRIPE_PRICE_IDS.PLUS_MONTHLY)`. STRIPE_PRICE_PLUS_MONTHLY is ABSENT from the local .env and .env.local; the Vercel production env cannot be read from here and AUTO-004 is blocked, so whether it is set live is STILL UNKNOWN -- and no unauthenticated probe can settle it, because create-checkout 401s before plan validation (see AUTO-009). If it is unset in production, every signed-in customer clicking Choose Plus gets a 400 'Invalid plan selected' and a signed-out one is routed through /register?plan=plus to the same dead end, on a page ads point at. ACTION FOR SRI, unchanged and now 1 day older: check that one env var in Vercel first. The fix either way is to gate the Plus card and CTA on isPlusPurchasable() and the report card on isReportPurchasable(), which is what those functions were written for. Separately app/api/billing/checkout/route.ts's ALLOWED_PRICE_IDS was never extended for Plus either. (2) STILL FAILING, 7th consecutive run since 2026-08-22: components/landing/UseCases.tsx:24 renders 'Trusted by marketing teams, agencies, and brands worldwide' under a 'Built for Modern Enterprises' heading -- re-confirmed verbatim in the live homepage text this run, and it is again the ONLY claim the live sweep surfaced across all six public pages (the sweep covered SOC 2, ISO 27001, HIPAA, uptime, awards, '#1', industry-leading, certified, patented, proven, guarantee and social-proof phrasing). Unverifiable social proof (plural teams, agencies, brands, worldwide); the last actual customer reading, 2026-08-29, was 1 active subscription. Not safely auto-fixable -- needs Sri to soften the copy. The only other sweep hit was /pricing's 'We do not guarantee rankings, mentions, or customer outcomes', which is a disclaimer and the opposite of a fabricated claim. (3) STILL DORMANT: components/landing/TrustBadges.tsx retains 'SOC 2 Compliant', '99.9% Uptime', '10M+ Keywords Analyzed Daily', '500+ Enterprises'. grep finds the identifier only in its own definition file -- zero imports -- and none of the four strings appear in the live HTML of any public page. Still needs a user-run rm; the sandbox cannot delete files. (4) STILL LATENT, the last dead-config trap: lib/seo-config.ts pages.dashboard survives untouched and still promises 'monitoring rankings, analyzing SERP performance, and measuring AI search visibility. Real-time SEO analytics' with a canonical at https://www.shijo.ai/dashboard -- an auth-gated route that must never be a canonical target. pages.features and pages.pricing were correctly rewritten on 2026-08-31 and now match real pages; pages.dashboard is the one that got left. Nothing renders it today, but one generatePageMetadata('dashboard') call publishes it. Recommend deleting the entry. (5) MINOR, unchanged: app/page.tsx JSON-LD offerCount is still '3' with a comment reading 'Free, Standard and Pro are purchasable' while four plans are advertised on the page; highPrice '199' is still correct and aggregateRating is still correctly absent. app/ai-marketing-tools/page.tsx has the same offerCount 3, which is accurate there since that page omits Plus. (6) UNRESOLVED, unchanged: /features:75 and /geo:48 both say 'We ask five answer engines' and the GEO UI hardcodes five, while only ANTHROPIC_API_KEY is present locally -- OPENAI_API_KEY, GEMINI_API_KEY, PERPLEXITY_API_KEY, DATAFORSEO_LOGIN and GOOGLE_PLACES_API_KEY are all absent from .env/.env.local. Production env is in Vercel and unreadable from here, and running a live scan to find out would spend real vendor credits, so this is still NOT confirmed as a production defect. Mitigating: lib/geo/orchestrator.ts degrades properly, recording unavailable engines as 'skipped' rather than scoring them as negatives. Before further ad spend on /geo, confirm all five keys exist in production or make the count dynamic. (7) CLEAN: app/layout.tsx metadata describes the real 12-tool product and claims no certifications.</t>
+        </is>
+      </c>
+      <c r="E169" s="7" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>

</xml_diff>